<commit_message>
Reduce false positive rent extraction
Co-authored-by: russlle2 <russlle2@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/income_based_housing_research_FL/housing_results.xlsx
+++ b/income_based_housing_research_FL/housing_results.xlsx
@@ -786,12 +786,12 @@
       </c>
       <c r="U2" s="2" t="inlineStr">
         <is>
-          <t>$1558; $1638; $1857; $2362; $2849</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="V2" s="2" t="inlineStr">
         <is>
-          <t>Published amounts appear to be maximum restricted LIHTC rents; confirm actual tenant rent with property.</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="W2" s="2" t="inlineStr">
@@ -892,7 +892,7 @@
         </is>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>0</v>
@@ -1192,12 +1192,12 @@
       </c>
       <c r="U4" s="2" t="inlineStr">
         <is>
-          <t>$1558; $1638; $1857; $2362; $2849</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="V4" s="2" t="inlineStr">
         <is>
-          <t>Published amounts appear to be maximum restricted LIHTC rents; confirm actual tenant rent with property.</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="W4" s="2" t="inlineStr">
@@ -1298,7 +1298,7 @@
         </is>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>0</v>
@@ -1403,12 +1403,12 @@
       </c>
       <c r="U5" s="2" t="inlineStr">
         <is>
-          <t>$945; $951; $1250; $1572; $1665</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="V5" s="2" t="inlineStr">
         <is>
-          <t>Published amounts appear to be maximum restricted LIHTC rents; confirm actual tenant rent with property.</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="W5" s="2" t="inlineStr">
@@ -1509,7 +1509,7 @@
         </is>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>5.7</v>
@@ -1598,12 +1598,12 @@
       </c>
       <c r="U6" s="2" t="inlineStr">
         <is>
-          <t>$1558; $1638; $1857; $2362; $2849</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="V6" s="2" t="inlineStr">
         <is>
-          <t>Published amounts appear to be maximum restricted LIHTC rents; confirm actual tenant rent with property.</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="W6" s="2" t="inlineStr">
@@ -1704,7 +1704,7 @@
         </is>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="AS6" s="2" t="n">
         <v>0</v>
@@ -1809,12 +1809,12 @@
       </c>
       <c r="U7" s="2" t="inlineStr">
         <is>
-          <t>$945; $951; $1250; $1572; $1665</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="V7" s="2" t="inlineStr">
         <is>
-          <t>Published amounts appear to be maximum restricted LIHTC rents; confirm actual tenant rent with property.</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="W7" s="2" t="inlineStr">
@@ -1915,7 +1915,7 @@
         </is>
       </c>
       <c r="AR7" s="2" t="n">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="AS7" s="2" t="n">
         <v>0</v>
@@ -2012,12 +2012,12 @@
       </c>
       <c r="U8" s="2" t="inlineStr">
         <is>
-          <t>$1558; $1638; $18; $1857; $2362; $2849</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="V8" s="2" t="inlineStr">
         <is>
-          <t>Published amounts appear to be maximum restricted LIHTC rents; confirm actual tenant rent with property.</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="W8" s="2" t="inlineStr">
@@ -2118,34 +2118,34 @@
         </is>
       </c>
       <c r="AR8" s="2" t="n">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="AS8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Panasoffkee Family Apartments</t>
+          <t>Lakeview Villas LTD</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Family</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>910 CR 482N</t>
+          <t>200 12th St Clermont</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Lake Panasoffkee</t>
+          <t>Clermont</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Sumter County</t>
+          <t>Lake County</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -2153,46 +2153,30 @@
           <t>FL</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>33538</t>
-        </is>
-      </c>
+      <c r="G9" s="2" t="inlineStr"/>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>(352) 793-2288</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>LowIncomeSupport@gmail.com</t>
-        </is>
-      </c>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>https://www.uslowcosthousing.com/foreclosure-housing/fl/lady_lake/fl-lady_lake-panasoffkee-family-apartments/</t>
-        </is>
-      </c>
+          <t>1 (352) 394-2896</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr"/>
+      <c r="J9" s="2" t="inlineStr"/>
       <c r="K9" s="2" t="inlineStr"/>
       <c r="L9" s="2" t="inlineStr"/>
-      <c r="M9" s="2" t="inlineStr">
-        <is>
-          <t>Sumter County Housing</t>
-        </is>
-      </c>
+      <c r="M9" s="2" t="inlineStr"/>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>https://www.sumtercountyfl.gov/246/Rental-Assistance-Resources; https://www.sumtercountyfl.gov/DocumentCenter/View/29964/Sumter-County-Multifamily-Analysis-Final-Version-06202018; https://sumtercountyfl.gov/246/Rental-Assistance-Resources; https://www.lowincomehousing.us/FL/lake_panasoffkee.html; https://www.lowincomehousing.us/FL/sumterville.html; https://www.uslowcosthousing.com/foreclosure-housing/fl/lady_lake/fl-lady_lake-panasoffkee-family-apartments/; https://www.uslowcosthousing.com/foreclosure-housing/fl/sanford/fl-sanford-overlook-at-monroe-apartments/; https://www.lowincomehousing.us/FL/center_hill.html</t>
+          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://www.publichousing.com/city/fl-clermont</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>government</t>
+          <t>HUD/USDA/FHFC</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>1 bedroom, 2 bedroom, 3 bedroom</t>
+          <t>1 bedroom</t>
         </is>
       </c>
       <c r="Q9" s="2" t="inlineStr"/>
@@ -2203,17 +2187,17 @@
       </c>
       <c r="S9" s="2" t="inlineStr">
         <is>
-          <t>Unknown affordable rental</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="T9" s="2" t="inlineStr">
         <is>
-          <t>income-based</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="U9" s="2" t="inlineStr">
         <is>
-          <t>$48,400; $88,300; $59,500</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="V9" s="2" t="inlineStr">
@@ -2258,7 +2242,7 @@
       </c>
       <c r="AD9" s="2" t="inlineStr">
         <is>
-          <t>Published credit-related language found; property verification recommended.</t>
+          <t>NOT FOUND / NEEDS CALL</t>
         </is>
       </c>
       <c r="AE9" s="2" t="inlineStr">
@@ -2311,35 +2295,33 @@
       </c>
       <c r="AQ9" s="2" t="inlineStr">
         <is>
-          <t>County multifamily inventory indicates family-focused property at same site as senior apartments. | Lake Panasoffkee Apartments - 352-793-2288</t>
+          <t>Lakeview Villas LTD | Clermont</t>
         </is>
       </c>
       <c r="AR9" s="2" t="n">
-        <v>87</v>
-      </c>
-      <c r="AS9" s="2" t="n">
-        <v>0</v>
-      </c>
+        <v>84</v>
+      </c>
+      <c r="AS9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Lakeview Villas LTD</t>
+          <t>Mirror Lake Manor</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>USDA RD</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>200 12th St Clermont</t>
+          <t>301 East Mirror Lk Fruitland Park</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Clermont</t>
+          <t>Fruitland Park</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -2355,7 +2337,7 @@
       <c r="G10" s="2" t="inlineStr"/>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>1 (352) 394-2896</t>
+          <t>1 352-728-4208</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr"/>
@@ -2365,7 +2347,7 @@
       <c r="M10" s="2" t="inlineStr"/>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://www.publichousing.com/city/fl-clermont</t>
+          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://www.publichousing.com/city/fl-fruitland_park</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
@@ -2373,25 +2355,21 @@
           <t>HUD/USDA/FHFC</t>
         </is>
       </c>
-      <c r="P10" s="2" t="inlineStr">
-        <is>
-          <t>1 bedroom</t>
-        </is>
-      </c>
+      <c r="P10" s="2" t="inlineStr"/>
       <c r="Q10" s="2" t="inlineStr"/>
       <c r="R10" s="2" t="inlineStr">
         <is>
-          <t>senior</t>
+          <t>disabled</t>
         </is>
       </c>
       <c r="S10" s="2" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>USDA RD 515</t>
         </is>
       </c>
       <c r="T10" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>income-based</t>
         </is>
       </c>
       <c r="U10" s="2" t="inlineStr">
@@ -2401,7 +2379,7 @@
       </c>
       <c r="V10" s="2" t="inlineStr">
         <is>
-          <t>NOT FOUND</t>
+          <t>Likely based on adjusted income; exact tenant rent requires application/property verification.</t>
         </is>
       </c>
       <c r="W10" s="2" t="inlineStr">
@@ -2494,33 +2472,35 @@
       </c>
       <c r="AQ10" s="2" t="inlineStr">
         <is>
-          <t>Lakeview Villas LTD | Clermont</t>
+          <t>Listed on USDA Rural Development Lake County property list. | Mirror Lake Manor | Fruitland Park Dr. | Mirror Lake Manor | Fruitland Park Dr. | Mirror Lake Manor | Fruitland Park Dr. | Mirror Lake Manor | Fruitland Park Dr. | Mirror Lake Manor | Fruitland Park Dr.</t>
         </is>
       </c>
       <c r="AR10" s="2" t="n">
         <v>84</v>
       </c>
-      <c r="AS10" s="2" t="inlineStr"/>
+      <c r="AS10" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Mirror Lake Manor</t>
+          <t>Pendry Villas</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>USDA RD</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>301 East Mirror Lk Fruitland Park</t>
+          <t>1303 2400 Kurt St</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Fruitland Park</t>
+          <t>Eustis</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -2536,7 +2516,7 @@
       <c r="G11" s="2" t="inlineStr"/>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>1 352-728-4208</t>
+          <t>(352) 357-3434</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr"/>
@@ -2546,7 +2526,7 @@
       <c r="M11" s="2" t="inlineStr"/>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://www.publichousing.com/city/fl-fruitland_park</t>
+          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://eustischamber.org/AboutEustis/housing.asp</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
@@ -2554,21 +2534,29 @@
           <t>HUD/USDA/FHFC</t>
         </is>
       </c>
-      <c r="P11" s="2" t="inlineStr"/>
-      <c r="Q11" s="2" t="inlineStr"/>
+      <c r="P11" s="2" t="inlineStr">
+        <is>
+          <t>4 bedroom, 4 bedrooms, 2 bedrooms, 3 bedrooms</t>
+        </is>
+      </c>
+      <c r="Q11" s="2" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
+      </c>
       <c r="R11" s="2" t="inlineStr">
         <is>
-          <t>disabled</t>
+          <t>senior</t>
         </is>
       </c>
       <c r="S11" s="2" t="inlineStr">
         <is>
-          <t>USDA RD 515</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="T11" s="2" t="inlineStr">
         <is>
-          <t>income-based</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="U11" s="2" t="inlineStr">
@@ -2578,7 +2566,7 @@
       </c>
       <c r="V11" s="2" t="inlineStr">
         <is>
-          <t>Likely based on adjusted income; exact tenant rent requires application/property verification.</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="W11" s="2" t="inlineStr">
@@ -2608,7 +2596,7 @@
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
-          <t>NOT FOUND / NEEDS CALL</t>
+          <t>Published pet-related language found; property verification recommended.</t>
         </is>
       </c>
       <c r="AC11" s="2" t="inlineStr">
@@ -2618,7 +2606,7 @@
       </c>
       <c r="AD11" s="2" t="inlineStr">
         <is>
-          <t>NOT FOUND / NEEDS CALL</t>
+          <t>Published credit-related language found; property verification recommended.</t>
         </is>
       </c>
       <c r="AE11" s="2" t="inlineStr">
@@ -2671,40 +2659,38 @@
       </c>
       <c r="AQ11" s="2" t="inlineStr">
         <is>
-          <t>Listed on USDA Rural Development Lake County property list. | Mirror Lake Manor | Fruitland Park Dr. | Mirror Lake Manor | Fruitland Park Dr. | Mirror Lake Manor | Fruitland Park Dr. | Mirror Lake Manor | Fruitland Park Dr. | Mirror Lake Manor | Fruitland Park Dr.</t>
+          <t>Pendry Villas | Eustis</t>
         </is>
       </c>
       <c r="AR11" s="2" t="n">
         <v>84</v>
       </c>
-      <c r="AS11" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="AS11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Pendry Villas</t>
+          <t>Panasoffkee Family Apartments</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Family</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>1303 2400 Kurt St</t>
+          <t>910 CR 482N</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Eustis</t>
+          <t>Lake Panasoffkee</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Lake County</t>
+          <t>Sumter County</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -2712,37 +2698,49 @@
           <t>FL</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr"/>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>33538</t>
+        </is>
+      </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>(352) 357-3434</t>
-        </is>
-      </c>
-      <c r="I12" s="2" t="inlineStr"/>
-      <c r="J12" s="2" t="inlineStr"/>
+          <t>(352) 793-2288</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>LowIncomeSupport@gmail.com</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>https://www.uslowcosthousing.com/foreclosure-housing/fl/lady_lake/fl-lady_lake-panasoffkee-family-apartments/</t>
+        </is>
+      </c>
       <c r="K12" s="2" t="inlineStr"/>
       <c r="L12" s="2" t="inlineStr"/>
-      <c r="M12" s="2" t="inlineStr"/>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>Sumter County Housing</t>
+        </is>
+      </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://eustischamber.org/AboutEustis/housing.asp</t>
+          <t>https://www.sumtercountyfl.gov/246/Rental-Assistance-Resources; https://www.sumtercountyfl.gov/DocumentCenter/View/29964/Sumter-County-Multifamily-Analysis-Final-Version-06202018; https://sumtercountyfl.gov/246/Rental-Assistance-Resources; https://www.lowincomehousing.us/FL/lake_panasoffkee.html; https://www.lowincomehousing.us/FL/sumterville.html; https://www.uslowcosthousing.com/foreclosure-housing/fl/lady_lake/fl-lady_lake-panasoffkee-family-apartments/; https://www.uslowcosthousing.com/foreclosure-housing/fl/sanford/fl-sanford-overlook-at-monroe-apartments/; https://www.lowincomehousing.us/FL/center_hill.html</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>HUD/USDA/FHFC</t>
+          <t>government</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>4 bedroom, 4 bedrooms, 2 bedrooms, 3 bedrooms</t>
-        </is>
-      </c>
-      <c r="Q12" s="2" t="inlineStr">
-        <is>
-          <t>47</t>
-        </is>
-      </c>
+          <t>1 bedroom, 2 bedroom, 3 bedroom</t>
+        </is>
+      </c>
+      <c r="Q12" s="2" t="inlineStr"/>
       <c r="R12" s="2" t="inlineStr">
         <is>
           <t>senior</t>
@@ -2750,12 +2748,12 @@
       </c>
       <c r="S12" s="2" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Unknown affordable rental</t>
         </is>
       </c>
       <c r="T12" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>income-based</t>
         </is>
       </c>
       <c r="U12" s="2" t="inlineStr">
@@ -2765,7 +2763,7 @@
       </c>
       <c r="V12" s="2" t="inlineStr">
         <is>
-          <t>NOT FOUND</t>
+          <t>Likely based on adjusted income; exact tenant rent requires application/property verification.</t>
         </is>
       </c>
       <c r="W12" s="2" t="inlineStr">
@@ -2795,7 +2793,7 @@
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
-          <t>Published pet-related language found; property verification recommended.</t>
+          <t>NOT FOUND / NEEDS CALL</t>
         </is>
       </c>
       <c r="AC12" s="2" t="inlineStr">
@@ -2858,13 +2856,15 @@
       </c>
       <c r="AQ12" s="2" t="inlineStr">
         <is>
-          <t>Pendry Villas | Eustis</t>
+          <t>County multifamily inventory indicates family-focused property at same site as senior apartments. | Lake Panasoffkee Apartments - 352-793-2288</t>
         </is>
       </c>
       <c r="AR12" s="2" t="n">
-        <v>84</v>
-      </c>
-      <c r="AS12" s="2" t="inlineStr"/>
+        <v>83</v>
+      </c>
+      <c r="AS12" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -4534,27 +4534,27 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Bushnell Garden Apartments</t>
+          <t>Fruitland Acres LTD</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>USDA RD</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>200 Jumper St S</t>
+          <t>303 Urick St</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Bushnell</t>
+          <t>Fruitland Park</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Sumter County</t>
+          <t>Lake County</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -4562,76 +4562,64 @@
           <t>FL</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr">
-        <is>
-          <t>33513</t>
-        </is>
-      </c>
+      <c r="G22" s="2" t="inlineStr"/>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>(352) 793-4838</t>
-        </is>
-      </c>
-      <c r="I22" s="2" t="inlineStr">
-        <is>
-          <t>LowIncomeSupport@gmail.com</t>
-        </is>
-      </c>
+          <t>(352) 323-3303</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr"/>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>https://affordablehousingonline.com/housing-search/Florida/Bushnell/Bushnell-Garden-Apartments/10000207</t>
+          <t>https://affordablehousingonline.com/housing-search/Florida/Fruitland-Park/Fruitland-Acres-Ltd/10026305</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>manges Bushnell Garden Apartments? Bushnell Garden Apartments is managed by Hale Management Group headquartered in Gainesville, Florida</t>
+          <t>private/corporate owners or nonprofits</t>
         </is>
       </c>
       <c r="L22" s="2" t="inlineStr"/>
-      <c r="M22" s="2" t="inlineStr">
-        <is>
-          <t>Sumter County Housing</t>
-        </is>
-      </c>
+      <c r="M22" s="2" t="inlineStr"/>
       <c r="N22" s="2" t="inlineStr">
         <is>
-          <t>https://www.sumtercountyfl.gov/246/Rental-Assistance-Resources; https://www.sumtercountyfl.gov/DocumentCenter/View/29964/Sumter-County-Multifamily-Analysis-Final-Version-06202018; https://sumtercountyfl.gov/246/Rental-Assistance-Resources; https://affordablehousingonline.com/housing-search/Florida/Bushnell/Bushnell-Garden-Apartments/10000207; https://www.lowincomehousing.us/FL/bushnell.html</t>
+          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://affordablehousingonline.com/housing-search/Florida/Fruitland-Park/Fruitland-Acres-Ltd/10026305; https://affordablehousingonline.com/housing-search/Florida/Fruitland-Park; https://affordablehousingonline.com/housing-search/Florida/Fruitland-Park/Mirror-Lake-Manor/10048622</t>
         </is>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>government</t>
+          <t>HUD/USDA/FHFC</t>
         </is>
       </c>
       <c r="P22" s="2" t="inlineStr">
         <is>
-          <t>3 Beds</t>
+          <t>2 Bed</t>
         </is>
       </c>
       <c r="Q22" s="2" t="inlineStr"/>
       <c r="R22" s="2" t="inlineStr">
         <is>
-          <t>senior</t>
+          <t>general low-income</t>
         </is>
       </c>
       <c r="S22" s="2" t="inlineStr">
         <is>
-          <t>Unknown affordable rental</t>
+          <t>USDA RD 515</t>
         </is>
       </c>
       <c r="T22" s="2" t="inlineStr">
         <is>
-          <t>fixed affordable rent</t>
+          <t>income-based</t>
         </is>
       </c>
       <c r="U22" s="2" t="inlineStr">
         <is>
-          <t>$600; $811; $700; $917; $775; $999</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="V22" s="2" t="inlineStr">
         <is>
-          <t>NOT FOUND</t>
+          <t>Likely based on adjusted income; exact tenant rent requires application/property verification.</t>
         </is>
       </c>
       <c r="W22" s="2" t="inlineStr">
@@ -4661,7 +4649,7 @@
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
-          <t>Published pet-related language found; property verification recommended.</t>
+          <t>NOT FOUND / NEEDS CALL</t>
         </is>
       </c>
       <c r="AC22" s="2" t="inlineStr">
@@ -4724,20 +4712,20 @@
       </c>
       <c r="AQ22" s="2" t="inlineStr">
         <is>
-          <t>Outside primary city list but near the target areas and listed by Sumter County as rental assistance provider. | Bushnell Garden Apartments - 352-793-4838</t>
+          <t>Listed on USDA Rural Development Lake County property list.</t>
         </is>
       </c>
       <c r="AR22" s="2" t="n">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="AS22" s="2" t="n">
-        <v>5.7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Fruitland Acres LTD</t>
+          <t>Montclair Village</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -4747,12 +4735,12 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>303 Urick St</t>
+          <t>2000 Park Cir</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Fruitland Park</t>
+          <t>Leesburg</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
@@ -4766,27 +4754,19 @@
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr"/>
-      <c r="H23" s="2" t="inlineStr">
-        <is>
-          <t>(352) 323-3303</t>
-        </is>
-      </c>
+      <c r="H23" s="2" t="inlineStr"/>
       <c r="I23" s="2" t="inlineStr"/>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>https://affordablehousingonline.com/housing-search/Florida/Fruitland-Park/Fruitland-Acres-Ltd/10026305</t>
-        </is>
-      </c>
-      <c r="K23" s="2" t="inlineStr">
-        <is>
-          <t>private/corporate owners or nonprofits</t>
-        </is>
-      </c>
+          <t>https://affordablehousingonline.com/housing-search/Florida/Leesburg/Montclair-Village/10103948</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr"/>
       <c r="L23" s="2" t="inlineStr"/>
       <c r="M23" s="2" t="inlineStr"/>
       <c r="N23" s="2" t="inlineStr">
         <is>
-          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://affordablehousingonline.com/housing-search/Florida/Fruitland-Park/Fruitland-Acres-Ltd/10026305; https://affordablehousingonline.com/housing-search/Florida/Fruitland-Park; https://affordablehousingonline.com/housing-search/Florida/Fruitland-Park/Mirror-Lake-Manor/10048622</t>
+          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://affordablehousingonline.com/housing-search/Florida/Leesburg/Montclair-Village/10103948; https://affordablehousingonline.com/housing-search/Florida/Leesburg</t>
         </is>
       </c>
       <c r="O23" s="2" t="inlineStr">
@@ -4802,7 +4782,7 @@
       <c r="Q23" s="2" t="inlineStr"/>
       <c r="R23" s="2" t="inlineStr">
         <is>
-          <t>general low-income</t>
+          <t>senior</t>
         </is>
       </c>
       <c r="S23" s="2" t="inlineStr">
@@ -4928,7 +4908,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Montclair Village</t>
+          <t>Palm Brook Apts LTD</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -4938,7 +4918,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>2000 Park Cir</t>
+          <t>37 Brook Cir</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -4961,15 +4941,19 @@
       <c r="I24" s="2" t="inlineStr"/>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>https://affordablehousingonline.com/housing-search/Florida/Leesburg/Montclair-Village/10103948</t>
-        </is>
-      </c>
-      <c r="K24" s="2" t="inlineStr"/>
+          <t>https://affordablehousingonline.com/housing-search/Florida/Leesburg/Palm-Brook-Apts-Ltd/10103487</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>private/corporate owners or nonprofits</t>
+        </is>
+      </c>
       <c r="L24" s="2" t="inlineStr"/>
       <c r="M24" s="2" t="inlineStr"/>
       <c r="N24" s="2" t="inlineStr">
         <is>
-          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://affordablehousingonline.com/housing-search/Florida/Leesburg/Montclair-Village/10103948; https://affordablehousingonline.com/housing-search/Florida/Leesburg</t>
+          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://affordablehousingonline.com/housing-search/Florida/Leesburg/Palm-Brook-Apts-Ltd/10103487; https://affordablehousingonline.com/housing-search/Florida/Leesburg</t>
         </is>
       </c>
       <c r="O24" s="2" t="inlineStr">
@@ -5111,7 +5095,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Palm Brook Apts LTD</t>
+          <t>Pepper Tree Apts</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -5121,7 +5105,7 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>37 Brook Cir</t>
+          <t>2503 South Street</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -5144,7 +5128,7 @@
       <c r="I25" s="2" t="inlineStr"/>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>https://affordablehousingonline.com/housing-search/Florida/Leesburg/Palm-Brook-Apts-Ltd/10103487</t>
+          <t>https://affordablehousingonline.com/housing-search/Florida/Leesburg/Pepper-Tree-Apts/10103485</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
@@ -5156,7 +5140,7 @@
       <c r="M25" s="2" t="inlineStr"/>
       <c r="N25" s="2" t="inlineStr">
         <is>
-          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://affordablehousingonline.com/housing-search/Florida/Leesburg/Palm-Brook-Apts-Ltd/10103487; https://affordablehousingonline.com/housing-search/Florida/Leesburg</t>
+          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://affordablehousingonline.com/housing-search/Florida/Leesburg/Pepper-Tree-Apts/10103485; https://affordablehousingonline.com/housing-search/Florida/Leesburg</t>
         </is>
       </c>
       <c r="O25" s="2" t="inlineStr">
@@ -5298,7 +5282,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Pepper Tree Apts</t>
+          <t>Pepper Tree Apts II</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -5331,7 +5315,7 @@
       <c r="I26" s="2" t="inlineStr"/>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>https://affordablehousingonline.com/housing-search/Florida/Leesburg/Pepper-Tree-Apts/10103485</t>
+          <t>https://affordablehousingonline.com/housing-search/Florida/Leesburg/Pepper-Tree-Apts-II/10104710</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr">
@@ -5343,7 +5327,7 @@
       <c r="M26" s="2" t="inlineStr"/>
       <c r="N26" s="2" t="inlineStr">
         <is>
-          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://affordablehousingonline.com/housing-search/Florida/Leesburg/Pepper-Tree-Apts/10103485; https://affordablehousingonline.com/housing-search/Florida/Leesburg</t>
+          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://affordablehousingonline.com/housing-search/Florida/Leesburg/Pepper-Tree-Apts-II/10104710; https://affordablehousingonline.com/housing-search/Florida/Leesburg</t>
         </is>
       </c>
       <c r="O26" s="2" t="inlineStr">
@@ -5485,27 +5469,27 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Pepper Tree Apts II</t>
+          <t>Bushnell Garden Apartments</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>USDA RD</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>2503 South Street</t>
+          <t>200 Jumper St S</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Leesburg</t>
+          <t>Bushnell</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Lake County</t>
+          <t>Sumter County</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
@@ -5513,34 +5497,50 @@
           <t>FL</t>
         </is>
       </c>
-      <c r="G27" s="2" t="inlineStr"/>
-      <c r="H27" s="2" t="inlineStr"/>
-      <c r="I27" s="2" t="inlineStr"/>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>33513</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>(352) 793-4838</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>LowIncomeSupport@gmail.com</t>
+        </is>
+      </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>https://affordablehousingonline.com/housing-search/Florida/Leesburg/Pepper-Tree-Apts-II/10104710</t>
+          <t>https://affordablehousingonline.com/housing-search/Florida/Bushnell/Bushnell-Garden-Apartments/10000207</t>
         </is>
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t>private/corporate owners or nonprofits</t>
+          <t>manges Bushnell Garden Apartments? Bushnell Garden Apartments is managed by Hale Management Group headquartered in Gainesville, Florida</t>
         </is>
       </c>
       <c r="L27" s="2" t="inlineStr"/>
-      <c r="M27" s="2" t="inlineStr"/>
+      <c r="M27" s="2" t="inlineStr">
+        <is>
+          <t>Sumter County Housing</t>
+        </is>
+      </c>
       <c r="N27" s="2" t="inlineStr">
         <is>
-          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://affordablehousingonline.com/housing-search/Florida/Leesburg/Pepper-Tree-Apts-II/10104710; https://affordablehousingonline.com/housing-search/Florida/Leesburg</t>
+          <t>https://www.sumtercountyfl.gov/246/Rental-Assistance-Resources; https://www.sumtercountyfl.gov/DocumentCenter/View/29964/Sumter-County-Multifamily-Analysis-Final-Version-06202018; https://sumtercountyfl.gov/246/Rental-Assistance-Resources; https://affordablehousingonline.com/housing-search/Florida/Bushnell/Bushnell-Garden-Apartments/10000207; https://www.lowincomehousing.us/FL/bushnell.html</t>
         </is>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t>HUD/USDA/FHFC</t>
+          <t>government</t>
         </is>
       </c>
       <c r="P27" s="2" t="inlineStr">
         <is>
-          <t>2 Bed</t>
+          <t>3 Beds</t>
         </is>
       </c>
       <c r="Q27" s="2" t="inlineStr"/>
@@ -5551,12 +5551,12 @@
       </c>
       <c r="S27" s="2" t="inlineStr">
         <is>
-          <t>USDA RD 515</t>
+          <t>Unknown affordable rental</t>
         </is>
       </c>
       <c r="T27" s="2" t="inlineStr">
         <is>
-          <t>income-based</t>
+          <t>fixed affordable rent</t>
         </is>
       </c>
       <c r="U27" s="2" t="inlineStr">
@@ -5566,7 +5566,7 @@
       </c>
       <c r="V27" s="2" t="inlineStr">
         <is>
-          <t>Likely based on adjusted income; exact tenant rent requires application/property verification.</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="W27" s="2" t="inlineStr">
@@ -5596,7 +5596,7 @@
       </c>
       <c r="AB27" s="2" t="inlineStr">
         <is>
-          <t>NOT FOUND / NEEDS CALL</t>
+          <t>Published pet-related language found; property verification recommended.</t>
         </is>
       </c>
       <c r="AC27" s="2" t="inlineStr">
@@ -5659,14 +5659,14 @@
       </c>
       <c r="AQ27" s="2" t="inlineStr">
         <is>
-          <t>Listed on USDA Rural Development Lake County property list.</t>
+          <t>Outside primary city list but near the target areas and listed by Sumter County as rental assistance provider. | Bushnell Garden Apartments - 352-793-4838</t>
         </is>
       </c>
       <c r="AR27" s="2" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AS27" s="2" t="n">
-        <v>0</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="28">
@@ -5744,12 +5744,12 @@
       </c>
       <c r="U28" s="2" t="inlineStr">
         <is>
-          <t>$911; $45,059; $152,928</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="V28" s="2" t="inlineStr">
         <is>
-          <t>NOT FOUND</t>
+          <t>Likely based on adjusted income; exact tenant rent requires application/property verification.</t>
         </is>
       </c>
       <c r="W28" s="2" t="inlineStr">
@@ -5850,7 +5850,7 @@
         </is>
       </c>
       <c r="AR28" s="2" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="AS28" s="2" t="n">
         <v>0</v>
@@ -5947,12 +5947,12 @@
       </c>
       <c r="U29" s="2" t="inlineStr">
         <is>
-          <t>$1558; $1638; $1857; $2362; $2849</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="V29" s="2" t="inlineStr">
         <is>
-          <t>Published amounts appear to be maximum restricted LIHTC rents; confirm actual tenant rent with property.</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="W29" s="2" t="inlineStr">
@@ -6053,7 +6053,7 @@
         </is>
       </c>
       <c r="AR29" s="2" t="n">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="AS29" s="2" t="inlineStr"/>
     </row>
@@ -6399,12 +6399,12 @@
       </c>
       <c r="U2" s="2" t="inlineStr">
         <is>
-          <t>$1558; $1638; $1857; $2362; $2849</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="V2" s="2" t="inlineStr">
         <is>
-          <t>Published amounts appear to be maximum restricted LIHTC rents; confirm actual tenant rent with property.</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="W2" s="2" t="inlineStr">
@@ -6505,7 +6505,7 @@
         </is>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>0</v>
@@ -6805,12 +6805,12 @@
       </c>
       <c r="U4" s="2" t="inlineStr">
         <is>
-          <t>$1558; $1638; $1857; $2362; $2849</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="V4" s="2" t="inlineStr">
         <is>
-          <t>Published amounts appear to be maximum restricted LIHTC rents; confirm actual tenant rent with property.</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="W4" s="2" t="inlineStr">
@@ -6911,7 +6911,7 @@
         </is>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>0</v>
@@ -7016,12 +7016,12 @@
       </c>
       <c r="U5" s="2" t="inlineStr">
         <is>
-          <t>$945; $951; $1250; $1572; $1665</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="V5" s="2" t="inlineStr">
         <is>
-          <t>Published amounts appear to be maximum restricted LIHTC rents; confirm actual tenant rent with property.</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="W5" s="2" t="inlineStr">
@@ -7122,7 +7122,7 @@
         </is>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>5.7</v>
@@ -7211,12 +7211,12 @@
       </c>
       <c r="U6" s="2" t="inlineStr">
         <is>
-          <t>$1558; $1638; $1857; $2362; $2849</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="V6" s="2" t="inlineStr">
         <is>
-          <t>Published amounts appear to be maximum restricted LIHTC rents; confirm actual tenant rent with property.</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="W6" s="2" t="inlineStr">
@@ -7317,7 +7317,7 @@
         </is>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="AS6" s="2" t="n">
         <v>0</v>
@@ -7422,12 +7422,12 @@
       </c>
       <c r="U7" s="2" t="inlineStr">
         <is>
-          <t>$945; $951; $1250; $1572; $1665</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="V7" s="2" t="inlineStr">
         <is>
-          <t>Published amounts appear to be maximum restricted LIHTC rents; confirm actual tenant rent with property.</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="W7" s="2" t="inlineStr">
@@ -7528,7 +7528,7 @@
         </is>
       </c>
       <c r="AR7" s="2" t="n">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="AS7" s="2" t="n">
         <v>0</v>
@@ -7625,12 +7625,12 @@
       </c>
       <c r="U8" s="2" t="inlineStr">
         <is>
-          <t>$1558; $1638; $18; $1857; $2362; $2849</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="V8" s="2" t="inlineStr">
         <is>
-          <t>Published amounts appear to be maximum restricted LIHTC rents; confirm actual tenant rent with property.</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="W8" s="2" t="inlineStr">
@@ -7731,7 +7731,7 @@
         </is>
       </c>
       <c r="AR8" s="2" t="n">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="AS8" s="2" t="inlineStr"/>
     </row>
@@ -8077,12 +8077,12 @@
       </c>
       <c r="U2" s="2" t="inlineStr">
         <is>
-          <t>$1558; $1638; $1857; $2362; $2849</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="V2" s="2" t="inlineStr">
         <is>
-          <t>Published amounts appear to be maximum restricted LIHTC rents; confirm actual tenant rent with property.</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="W2" s="2" t="inlineStr">
@@ -8183,7 +8183,7 @@
         </is>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>0</v>
@@ -8483,12 +8483,12 @@
       </c>
       <c r="U4" s="2" t="inlineStr">
         <is>
-          <t>$1558; $1638; $1857; $2362; $2849</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="V4" s="2" t="inlineStr">
         <is>
-          <t>Published amounts appear to be maximum restricted LIHTC rents; confirm actual tenant rent with property.</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="W4" s="2" t="inlineStr">
@@ -8589,7 +8589,7 @@
         </is>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>0</v>
@@ -8694,12 +8694,12 @@
       </c>
       <c r="U5" s="2" t="inlineStr">
         <is>
-          <t>$945; $951; $1250; $1572; $1665</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="V5" s="2" t="inlineStr">
         <is>
-          <t>Published amounts appear to be maximum restricted LIHTC rents; confirm actual tenant rent with property.</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="W5" s="2" t="inlineStr">
@@ -8800,7 +8800,7 @@
         </is>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>5.7</v>
@@ -8889,12 +8889,12 @@
       </c>
       <c r="U6" s="2" t="inlineStr">
         <is>
-          <t>$1558; $1638; $1857; $2362; $2849</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="V6" s="2" t="inlineStr">
         <is>
-          <t>Published amounts appear to be maximum restricted LIHTC rents; confirm actual tenant rent with property.</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="W6" s="2" t="inlineStr">
@@ -8995,7 +8995,7 @@
         </is>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="AS6" s="2" t="n">
         <v>0</v>
@@ -9100,12 +9100,12 @@
       </c>
       <c r="U7" s="2" t="inlineStr">
         <is>
-          <t>$945; $951; $1250; $1572; $1665</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="V7" s="2" t="inlineStr">
         <is>
-          <t>Published amounts appear to be maximum restricted LIHTC rents; confirm actual tenant rent with property.</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="W7" s="2" t="inlineStr">
@@ -9206,7 +9206,7 @@
         </is>
       </c>
       <c r="AR7" s="2" t="n">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="AS7" s="2" t="n">
         <v>0</v>
@@ -9303,12 +9303,12 @@
       </c>
       <c r="U8" s="2" t="inlineStr">
         <is>
-          <t>$1558; $1638; $18; $1857; $2362; $2849</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="V8" s="2" t="inlineStr">
         <is>
-          <t>Published amounts appear to be maximum restricted LIHTC rents; confirm actual tenant rent with property.</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="W8" s="2" t="inlineStr">
@@ -9409,34 +9409,34 @@
         </is>
       </c>
       <c r="AR8" s="2" t="n">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="AS8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Panasoffkee Family Apartments</t>
+          <t>Mirror Lake Manor</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Family</t>
+          <t>USDA RD</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>910 CR 482N</t>
+          <t>301 East Mirror Lk Fruitland Park</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Lake Panasoffkee</t>
+          <t>Fruitland Park</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Sumter County</t>
+          <t>Lake County</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -9444,57 +9444,37 @@
           <t>FL</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>33538</t>
-        </is>
-      </c>
+      <c r="G9" s="2" t="inlineStr"/>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>(352) 793-2288</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>LowIncomeSupport@gmail.com</t>
-        </is>
-      </c>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>https://www.uslowcosthousing.com/foreclosure-housing/fl/lady_lake/fl-lady_lake-panasoffkee-family-apartments/</t>
-        </is>
-      </c>
+          <t>1 352-728-4208</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr"/>
+      <c r="J9" s="2" t="inlineStr"/>
       <c r="K9" s="2" t="inlineStr"/>
       <c r="L9" s="2" t="inlineStr"/>
-      <c r="M9" s="2" t="inlineStr">
-        <is>
-          <t>Sumter County Housing</t>
-        </is>
-      </c>
+      <c r="M9" s="2" t="inlineStr"/>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>https://www.sumtercountyfl.gov/246/Rental-Assistance-Resources; https://www.sumtercountyfl.gov/DocumentCenter/View/29964/Sumter-County-Multifamily-Analysis-Final-Version-06202018; https://sumtercountyfl.gov/246/Rental-Assistance-Resources; https://www.lowincomehousing.us/FL/lake_panasoffkee.html; https://www.lowincomehousing.us/FL/sumterville.html; https://www.uslowcosthousing.com/foreclosure-housing/fl/lady_lake/fl-lady_lake-panasoffkee-family-apartments/; https://www.uslowcosthousing.com/foreclosure-housing/fl/sanford/fl-sanford-overlook-at-monroe-apartments/; https://www.lowincomehousing.us/FL/center_hill.html</t>
+          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://www.publichousing.com/city/fl-fruitland_park</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>government</t>
-        </is>
-      </c>
-      <c r="P9" s="2" t="inlineStr">
-        <is>
-          <t>1 bedroom, 2 bedroom, 3 bedroom</t>
-        </is>
-      </c>
+          <t>HUD/USDA/FHFC</t>
+        </is>
+      </c>
+      <c r="P9" s="2" t="inlineStr"/>
       <c r="Q9" s="2" t="inlineStr"/>
       <c r="R9" s="2" t="inlineStr">
         <is>
-          <t>senior</t>
+          <t>disabled</t>
         </is>
       </c>
       <c r="S9" s="2" t="inlineStr">
         <is>
-          <t>Unknown affordable rental</t>
+          <t>USDA RD 515</t>
         </is>
       </c>
       <c r="T9" s="2" t="inlineStr">
@@ -9504,12 +9484,12 @@
       </c>
       <c r="U9" s="2" t="inlineStr">
         <is>
-          <t>$48,400; $88,300; $59,500</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="V9" s="2" t="inlineStr">
         <is>
-          <t>NOT FOUND</t>
+          <t>Likely based on adjusted income; exact tenant rent requires application/property verification.</t>
         </is>
       </c>
       <c r="W9" s="2" t="inlineStr">
@@ -9549,7 +9529,7 @@
       </c>
       <c r="AD9" s="2" t="inlineStr">
         <is>
-          <t>Published credit-related language found; property verification recommended.</t>
+          <t>NOT FOUND / NEEDS CALL</t>
         </is>
       </c>
       <c r="AE9" s="2" t="inlineStr">
@@ -9602,11 +9582,11 @@
       </c>
       <c r="AQ9" s="2" t="inlineStr">
         <is>
-          <t>County multifamily inventory indicates family-focused property at same site as senior apartments. | Lake Panasoffkee Apartments - 352-793-2288</t>
+          <t>Listed on USDA Rural Development Lake County property list. | Mirror Lake Manor | Fruitland Park Dr. | Mirror Lake Manor | Fruitland Park Dr. | Mirror Lake Manor | Fruitland Park Dr. | Mirror Lake Manor | Fruitland Park Dr. | Mirror Lake Manor | Fruitland Park Dr.</t>
         </is>
       </c>
       <c r="AR9" s="2" t="n">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="AS9" s="2" t="n">
         <v>0</v>
@@ -9615,27 +9595,27 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Mirror Lake Manor</t>
+          <t>Panasoffkee Family Apartments</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>USDA RD</t>
+          <t>Family</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>301 East Mirror Lk Fruitland Park</t>
+          <t>910 CR 482N</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Fruitland Park</t>
+          <t>Lake Panasoffkee</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Lake County</t>
+          <t>Sumter County</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -9643,37 +9623,57 @@
           <t>FL</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr"/>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>33538</t>
+        </is>
+      </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>1 352-728-4208</t>
-        </is>
-      </c>
-      <c r="I10" s="2" t="inlineStr"/>
-      <c r="J10" s="2" t="inlineStr"/>
+          <t>(352) 793-2288</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>LowIncomeSupport@gmail.com</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>https://www.uslowcosthousing.com/foreclosure-housing/fl/lady_lake/fl-lady_lake-panasoffkee-family-apartments/</t>
+        </is>
+      </c>
       <c r="K10" s="2" t="inlineStr"/>
       <c r="L10" s="2" t="inlineStr"/>
-      <c r="M10" s="2" t="inlineStr"/>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>Sumter County Housing</t>
+        </is>
+      </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://www.publichousing.com/city/fl-fruitland_park</t>
+          <t>https://www.sumtercountyfl.gov/246/Rental-Assistance-Resources; https://www.sumtercountyfl.gov/DocumentCenter/View/29964/Sumter-County-Multifamily-Analysis-Final-Version-06202018; https://sumtercountyfl.gov/246/Rental-Assistance-Resources; https://www.lowincomehousing.us/FL/lake_panasoffkee.html; https://www.lowincomehousing.us/FL/sumterville.html; https://www.uslowcosthousing.com/foreclosure-housing/fl/lady_lake/fl-lady_lake-panasoffkee-family-apartments/; https://www.uslowcosthousing.com/foreclosure-housing/fl/sanford/fl-sanford-overlook-at-monroe-apartments/; https://www.lowincomehousing.us/FL/center_hill.html</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>HUD/USDA/FHFC</t>
-        </is>
-      </c>
-      <c r="P10" s="2" t="inlineStr"/>
+          <t>government</t>
+        </is>
+      </c>
+      <c r="P10" s="2" t="inlineStr">
+        <is>
+          <t>1 bedroom, 2 bedroom, 3 bedroom</t>
+        </is>
+      </c>
       <c r="Q10" s="2" t="inlineStr"/>
       <c r="R10" s="2" t="inlineStr">
         <is>
-          <t>disabled</t>
+          <t>senior</t>
         </is>
       </c>
       <c r="S10" s="2" t="inlineStr">
         <is>
-          <t>USDA RD 515</t>
+          <t>Unknown affordable rental</t>
         </is>
       </c>
       <c r="T10" s="2" t="inlineStr">
@@ -9728,7 +9728,7 @@
       </c>
       <c r="AD10" s="2" t="inlineStr">
         <is>
-          <t>NOT FOUND / NEEDS CALL</t>
+          <t>Published credit-related language found; property verification recommended.</t>
         </is>
       </c>
       <c r="AE10" s="2" t="inlineStr">
@@ -9781,11 +9781,11 @@
       </c>
       <c r="AQ10" s="2" t="inlineStr">
         <is>
-          <t>Listed on USDA Rural Development Lake County property list. | Mirror Lake Manor | Fruitland Park Dr. | Mirror Lake Manor | Fruitland Park Dr. | Mirror Lake Manor | Fruitland Park Dr. | Mirror Lake Manor | Fruitland Park Dr. | Mirror Lake Manor | Fruitland Park Dr.</t>
+          <t>County multifamily inventory indicates family-focused property at same site as senior apartments. | Lake Panasoffkee Apartments - 352-793-2288</t>
         </is>
       </c>
       <c r="AR10" s="2" t="n">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="AS10" s="2" t="n">
         <v>0</v>
@@ -10709,27 +10709,27 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Bushnell Garden Apartments</t>
+          <t>Fruitland Acres LTD</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>USDA RD</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>200 Jumper St S</t>
+          <t>303 Urick St</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Bushnell</t>
+          <t>Fruitland Park</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Sumter County</t>
+          <t>Lake County</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -10737,76 +10737,64 @@
           <t>FL</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>33513</t>
-        </is>
-      </c>
+      <c r="G16" s="2" t="inlineStr"/>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>(352) 793-4838</t>
-        </is>
-      </c>
-      <c r="I16" s="2" t="inlineStr">
-        <is>
-          <t>LowIncomeSupport@gmail.com</t>
-        </is>
-      </c>
+          <t>(352) 323-3303</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr"/>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>https://affordablehousingonline.com/housing-search/Florida/Bushnell/Bushnell-Garden-Apartments/10000207</t>
+          <t>https://affordablehousingonline.com/housing-search/Florida/Fruitland-Park/Fruitland-Acres-Ltd/10026305</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>manges Bushnell Garden Apartments? Bushnell Garden Apartments is managed by Hale Management Group headquartered in Gainesville, Florida</t>
+          <t>private/corporate owners or nonprofits</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr"/>
-      <c r="M16" s="2" t="inlineStr">
-        <is>
-          <t>Sumter County Housing</t>
-        </is>
-      </c>
+      <c r="M16" s="2" t="inlineStr"/>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>https://www.sumtercountyfl.gov/246/Rental-Assistance-Resources; https://www.sumtercountyfl.gov/DocumentCenter/View/29964/Sumter-County-Multifamily-Analysis-Final-Version-06202018; https://sumtercountyfl.gov/246/Rental-Assistance-Resources; https://affordablehousingonline.com/housing-search/Florida/Bushnell/Bushnell-Garden-Apartments/10000207; https://www.lowincomehousing.us/FL/bushnell.html</t>
+          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://affordablehousingonline.com/housing-search/Florida/Fruitland-Park/Fruitland-Acres-Ltd/10026305; https://affordablehousingonline.com/housing-search/Florida/Fruitland-Park; https://affordablehousingonline.com/housing-search/Florida/Fruitland-Park/Mirror-Lake-Manor/10048622</t>
         </is>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>government</t>
+          <t>HUD/USDA/FHFC</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>3 Beds</t>
+          <t>2 Bed</t>
         </is>
       </c>
       <c r="Q16" s="2" t="inlineStr"/>
       <c r="R16" s="2" t="inlineStr">
         <is>
-          <t>senior</t>
+          <t>general low-income</t>
         </is>
       </c>
       <c r="S16" s="2" t="inlineStr">
         <is>
-          <t>Unknown affordable rental</t>
+          <t>USDA RD 515</t>
         </is>
       </c>
       <c r="T16" s="2" t="inlineStr">
         <is>
-          <t>fixed affordable rent</t>
+          <t>income-based</t>
         </is>
       </c>
       <c r="U16" s="2" t="inlineStr">
         <is>
-          <t>$600; $811; $700; $917; $775; $999</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="V16" s="2" t="inlineStr">
         <is>
-          <t>NOT FOUND</t>
+          <t>Likely based on adjusted income; exact tenant rent requires application/property verification.</t>
         </is>
       </c>
       <c r="W16" s="2" t="inlineStr">
@@ -10836,7 +10824,7 @@
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
-          <t>Published pet-related language found; property verification recommended.</t>
+          <t>NOT FOUND / NEEDS CALL</t>
         </is>
       </c>
       <c r="AC16" s="2" t="inlineStr">
@@ -10899,20 +10887,20 @@
       </c>
       <c r="AQ16" s="2" t="inlineStr">
         <is>
-          <t>Outside primary city list but near the target areas and listed by Sumter County as rental assistance provider. | Bushnell Garden Apartments - 352-793-4838</t>
+          <t>Listed on USDA Rural Development Lake County property list.</t>
         </is>
       </c>
       <c r="AR16" s="2" t="n">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="AS16" s="2" t="n">
-        <v>5.7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Fruitland Acres LTD</t>
+          <t>Montclair Village</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -10922,12 +10910,12 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>303 Urick St</t>
+          <t>2000 Park Cir</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Fruitland Park</t>
+          <t>Leesburg</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -10941,27 +10929,19 @@
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr"/>
-      <c r="H17" s="2" t="inlineStr">
-        <is>
-          <t>(352) 323-3303</t>
-        </is>
-      </c>
+      <c r="H17" s="2" t="inlineStr"/>
       <c r="I17" s="2" t="inlineStr"/>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>https://affordablehousingonline.com/housing-search/Florida/Fruitland-Park/Fruitland-Acres-Ltd/10026305</t>
-        </is>
-      </c>
-      <c r="K17" s="2" t="inlineStr">
-        <is>
-          <t>private/corporate owners or nonprofits</t>
-        </is>
-      </c>
+          <t>https://affordablehousingonline.com/housing-search/Florida/Leesburg/Montclair-Village/10103948</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr"/>
       <c r="L17" s="2" t="inlineStr"/>
       <c r="M17" s="2" t="inlineStr"/>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://affordablehousingonline.com/housing-search/Florida/Fruitland-Park/Fruitland-Acres-Ltd/10026305; https://affordablehousingonline.com/housing-search/Florida/Fruitland-Park; https://affordablehousingonline.com/housing-search/Florida/Fruitland-Park/Mirror-Lake-Manor/10048622</t>
+          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://affordablehousingonline.com/housing-search/Florida/Leesburg/Montclair-Village/10103948; https://affordablehousingonline.com/housing-search/Florida/Leesburg</t>
         </is>
       </c>
       <c r="O17" s="2" t="inlineStr">
@@ -10977,7 +10957,7 @@
       <c r="Q17" s="2" t="inlineStr"/>
       <c r="R17" s="2" t="inlineStr">
         <is>
-          <t>general low-income</t>
+          <t>senior</t>
         </is>
       </c>
       <c r="S17" s="2" t="inlineStr">
@@ -11103,7 +11083,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Montclair Village</t>
+          <t>Palm Brook Apts LTD</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -11113,7 +11093,7 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>2000 Park Cir</t>
+          <t>37 Brook Cir</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -11136,15 +11116,19 @@
       <c r="I18" s="2" t="inlineStr"/>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>https://affordablehousingonline.com/housing-search/Florida/Leesburg/Montclair-Village/10103948</t>
-        </is>
-      </c>
-      <c r="K18" s="2" t="inlineStr"/>
+          <t>https://affordablehousingonline.com/housing-search/Florida/Leesburg/Palm-Brook-Apts-Ltd/10103487</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>private/corporate owners or nonprofits</t>
+        </is>
+      </c>
       <c r="L18" s="2" t="inlineStr"/>
       <c r="M18" s="2" t="inlineStr"/>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://affordablehousingonline.com/housing-search/Florida/Leesburg/Montclair-Village/10103948; https://affordablehousingonline.com/housing-search/Florida/Leesburg</t>
+          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://affordablehousingonline.com/housing-search/Florida/Leesburg/Palm-Brook-Apts-Ltd/10103487; https://affordablehousingonline.com/housing-search/Florida/Leesburg</t>
         </is>
       </c>
       <c r="O18" s="2" t="inlineStr">
@@ -11286,7 +11270,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Palm Brook Apts LTD</t>
+          <t>Pepper Tree Apts</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -11296,7 +11280,7 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>37 Brook Cir</t>
+          <t>2503 South Street</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -11319,7 +11303,7 @@
       <c r="I19" s="2" t="inlineStr"/>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>https://affordablehousingonline.com/housing-search/Florida/Leesburg/Palm-Brook-Apts-Ltd/10103487</t>
+          <t>https://affordablehousingonline.com/housing-search/Florida/Leesburg/Pepper-Tree-Apts/10103485</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
@@ -11331,7 +11315,7 @@
       <c r="M19" s="2" t="inlineStr"/>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://affordablehousingonline.com/housing-search/Florida/Leesburg/Palm-Brook-Apts-Ltd/10103487; https://affordablehousingonline.com/housing-search/Florida/Leesburg</t>
+          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://affordablehousingonline.com/housing-search/Florida/Leesburg/Pepper-Tree-Apts/10103485; https://affordablehousingonline.com/housing-search/Florida/Leesburg</t>
         </is>
       </c>
       <c r="O19" s="2" t="inlineStr">
@@ -11473,7 +11457,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Pepper Tree Apts</t>
+          <t>Pepper Tree Apts II</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -11506,7 +11490,7 @@
       <c r="I20" s="2" t="inlineStr"/>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>https://affordablehousingonline.com/housing-search/Florida/Leesburg/Pepper-Tree-Apts/10103485</t>
+          <t>https://affordablehousingonline.com/housing-search/Florida/Leesburg/Pepper-Tree-Apts-II/10104710</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
@@ -11518,7 +11502,7 @@
       <c r="M20" s="2" t="inlineStr"/>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://affordablehousingonline.com/housing-search/Florida/Leesburg/Pepper-Tree-Apts/10103485; https://affordablehousingonline.com/housing-search/Florida/Leesburg</t>
+          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://affordablehousingonline.com/housing-search/Florida/Leesburg/Pepper-Tree-Apts-II/10104710; https://affordablehousingonline.com/housing-search/Florida/Leesburg</t>
         </is>
       </c>
       <c r="O20" s="2" t="inlineStr">
@@ -11660,27 +11644,27 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Pepper Tree Apts II</t>
+          <t>Bushnell Garden Apartments</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>USDA RD</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>2503 South Street</t>
+          <t>200 Jumper St S</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Leesburg</t>
+          <t>Bushnell</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Lake County</t>
+          <t>Sumter County</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
@@ -11688,34 +11672,50 @@
           <t>FL</t>
         </is>
       </c>
-      <c r="G21" s="2" t="inlineStr"/>
-      <c r="H21" s="2" t="inlineStr"/>
-      <c r="I21" s="2" t="inlineStr"/>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>33513</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>(352) 793-4838</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>LowIncomeSupport@gmail.com</t>
+        </is>
+      </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>https://affordablehousingonline.com/housing-search/Florida/Leesburg/Pepper-Tree-Apts-II/10104710</t>
+          <t>https://affordablehousingonline.com/housing-search/Florida/Bushnell/Bushnell-Garden-Apartments/10000207</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>private/corporate owners or nonprofits</t>
+          <t>manges Bushnell Garden Apartments? Bushnell Garden Apartments is managed by Hale Management Group headquartered in Gainesville, Florida</t>
         </is>
       </c>
       <c r="L21" s="2" t="inlineStr"/>
-      <c r="M21" s="2" t="inlineStr"/>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>Sumter County Housing</t>
+        </is>
+      </c>
       <c r="N21" s="2" t="inlineStr">
         <is>
-          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://affordablehousingonline.com/housing-search/Florida/Leesburg/Pepper-Tree-Apts-II/10104710; https://affordablehousingonline.com/housing-search/Florida/Leesburg</t>
+          <t>https://www.sumtercountyfl.gov/246/Rental-Assistance-Resources; https://www.sumtercountyfl.gov/DocumentCenter/View/29964/Sumter-County-Multifamily-Analysis-Final-Version-06202018; https://sumtercountyfl.gov/246/Rental-Assistance-Resources; https://affordablehousingonline.com/housing-search/Florida/Bushnell/Bushnell-Garden-Apartments/10000207; https://www.lowincomehousing.us/FL/bushnell.html</t>
         </is>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>HUD/USDA/FHFC</t>
+          <t>government</t>
         </is>
       </c>
       <c r="P21" s="2" t="inlineStr">
         <is>
-          <t>2 Bed</t>
+          <t>3 Beds</t>
         </is>
       </c>
       <c r="Q21" s="2" t="inlineStr"/>
@@ -11726,12 +11726,12 @@
       </c>
       <c r="S21" s="2" t="inlineStr">
         <is>
-          <t>USDA RD 515</t>
+          <t>Unknown affordable rental</t>
         </is>
       </c>
       <c r="T21" s="2" t="inlineStr">
         <is>
-          <t>income-based</t>
+          <t>fixed affordable rent</t>
         </is>
       </c>
       <c r="U21" s="2" t="inlineStr">
@@ -11741,7 +11741,7 @@
       </c>
       <c r="V21" s="2" t="inlineStr">
         <is>
-          <t>Likely based on adjusted income; exact tenant rent requires application/property verification.</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="W21" s="2" t="inlineStr">
@@ -11771,7 +11771,7 @@
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
-          <t>NOT FOUND / NEEDS CALL</t>
+          <t>Published pet-related language found; property verification recommended.</t>
         </is>
       </c>
       <c r="AC21" s="2" t="inlineStr">
@@ -11834,14 +11834,14 @@
       </c>
       <c r="AQ21" s="2" t="inlineStr">
         <is>
-          <t>Listed on USDA Rural Development Lake County property list.</t>
+          <t>Outside primary city list but near the target areas and listed by Sumter County as rental assistance provider. | Bushnell Garden Apartments - 352-793-4838</t>
         </is>
       </c>
       <c r="AR21" s="2" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AS21" s="2" t="n">
-        <v>0</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="22">
@@ -11919,12 +11919,12 @@
       </c>
       <c r="U22" s="2" t="inlineStr">
         <is>
-          <t>$911; $45,059; $152,928</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="V22" s="2" t="inlineStr">
         <is>
-          <t>NOT FOUND</t>
+          <t>Likely based on adjusted income; exact tenant rent requires application/property verification.</t>
         </is>
       </c>
       <c r="W22" s="2" t="inlineStr">
@@ -12025,7 +12025,7 @@
         </is>
       </c>
       <c r="AR22" s="2" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="AS22" s="2" t="n">
         <v>0</v>
@@ -12122,12 +12122,12 @@
       </c>
       <c r="U23" s="2" t="inlineStr">
         <is>
-          <t>$1558; $1638; $1857; $2362; $2849</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="V23" s="2" t="inlineStr">
         <is>
-          <t>Published amounts appear to be maximum restricted LIHTC rents; confirm actual tenant rent with property.</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="W23" s="2" t="inlineStr">
@@ -12228,7 +12228,7 @@
         </is>
       </c>
       <c r="AR23" s="2" t="n">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="AS23" s="2" t="inlineStr"/>
     </row>
@@ -12574,12 +12574,12 @@
       </c>
       <c r="U2" s="2" t="inlineStr">
         <is>
-          <t>$1558; $1638; $1857; $2362; $2849</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="V2" s="2" t="inlineStr">
         <is>
-          <t>Published amounts appear to be maximum restricted LIHTC rents; confirm actual tenant rent with property.</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="W2" s="2" t="inlineStr">
@@ -12680,7 +12680,7 @@
         </is>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>0</v>
@@ -12980,12 +12980,12 @@
       </c>
       <c r="U4" s="2" t="inlineStr">
         <is>
-          <t>$1558; $1638; $1857; $2362; $2849</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="V4" s="2" t="inlineStr">
         <is>
-          <t>Published amounts appear to be maximum restricted LIHTC rents; confirm actual tenant rent with property.</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="W4" s="2" t="inlineStr">
@@ -13086,7 +13086,7 @@
         </is>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>0</v>
@@ -13191,12 +13191,12 @@
       </c>
       <c r="U5" s="2" t="inlineStr">
         <is>
-          <t>$945; $951; $1250; $1572; $1665</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="V5" s="2" t="inlineStr">
         <is>
-          <t>Published amounts appear to be maximum restricted LIHTC rents; confirm actual tenant rent with property.</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="W5" s="2" t="inlineStr">
@@ -13297,7 +13297,7 @@
         </is>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>5.7</v>
@@ -13386,12 +13386,12 @@
       </c>
       <c r="U6" s="2" t="inlineStr">
         <is>
-          <t>$1558; $1638; $1857; $2362; $2849</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="V6" s="2" t="inlineStr">
         <is>
-          <t>Published amounts appear to be maximum restricted LIHTC rents; confirm actual tenant rent with property.</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="W6" s="2" t="inlineStr">
@@ -13492,7 +13492,7 @@
         </is>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="AS6" s="2" t="n">
         <v>0</v>
@@ -13597,12 +13597,12 @@
       </c>
       <c r="U7" s="2" t="inlineStr">
         <is>
-          <t>$945; $951; $1250; $1572; $1665</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="V7" s="2" t="inlineStr">
         <is>
-          <t>Published amounts appear to be maximum restricted LIHTC rents; confirm actual tenant rent with property.</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="W7" s="2" t="inlineStr">
@@ -13703,7 +13703,7 @@
         </is>
       </c>
       <c r="AR7" s="2" t="n">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="AS7" s="2" t="n">
         <v>0</v>
@@ -13800,12 +13800,12 @@
       </c>
       <c r="U8" s="2" t="inlineStr">
         <is>
-          <t>$1558; $1638; $18; $1857; $2362; $2849</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="V8" s="2" t="inlineStr">
         <is>
-          <t>Published amounts appear to be maximum restricted LIHTC rents; confirm actual tenant rent with property.</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="W8" s="2" t="inlineStr">
@@ -13906,34 +13906,34 @@
         </is>
       </c>
       <c r="AR8" s="2" t="n">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="AS8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Panasoffkee Family Apartments</t>
+          <t>Lakeview Villas LTD</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Family</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>910 CR 482N</t>
+          <t>200 12th St Clermont</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Lake Panasoffkee</t>
+          <t>Clermont</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Sumter County</t>
+          <t>Lake County</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -13941,46 +13941,30 @@
           <t>FL</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>33538</t>
-        </is>
-      </c>
+      <c r="G9" s="2" t="inlineStr"/>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>(352) 793-2288</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>LowIncomeSupport@gmail.com</t>
-        </is>
-      </c>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>https://www.uslowcosthousing.com/foreclosure-housing/fl/lady_lake/fl-lady_lake-panasoffkee-family-apartments/</t>
-        </is>
-      </c>
+          <t>1 (352) 394-2896</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr"/>
+      <c r="J9" s="2" t="inlineStr"/>
       <c r="K9" s="2" t="inlineStr"/>
       <c r="L9" s="2" t="inlineStr"/>
-      <c r="M9" s="2" t="inlineStr">
-        <is>
-          <t>Sumter County Housing</t>
-        </is>
-      </c>
+      <c r="M9" s="2" t="inlineStr"/>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>https://www.sumtercountyfl.gov/246/Rental-Assistance-Resources; https://www.sumtercountyfl.gov/DocumentCenter/View/29964/Sumter-County-Multifamily-Analysis-Final-Version-06202018; https://sumtercountyfl.gov/246/Rental-Assistance-Resources; https://www.lowincomehousing.us/FL/lake_panasoffkee.html; https://www.lowincomehousing.us/FL/sumterville.html; https://www.uslowcosthousing.com/foreclosure-housing/fl/lady_lake/fl-lady_lake-panasoffkee-family-apartments/; https://www.uslowcosthousing.com/foreclosure-housing/fl/sanford/fl-sanford-overlook-at-monroe-apartments/; https://www.lowincomehousing.us/FL/center_hill.html</t>
+          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://www.publichousing.com/city/fl-clermont</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>government</t>
+          <t>HUD/USDA/FHFC</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>1 bedroom, 2 bedroom, 3 bedroom</t>
+          <t>1 bedroom</t>
         </is>
       </c>
       <c r="Q9" s="2" t="inlineStr"/>
@@ -13991,17 +13975,17 @@
       </c>
       <c r="S9" s="2" t="inlineStr">
         <is>
-          <t>Unknown affordable rental</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="T9" s="2" t="inlineStr">
         <is>
-          <t>income-based</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="U9" s="2" t="inlineStr">
         <is>
-          <t>$48,400; $88,300; $59,500</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="V9" s="2" t="inlineStr">
@@ -14046,7 +14030,7 @@
       </c>
       <c r="AD9" s="2" t="inlineStr">
         <is>
-          <t>Published credit-related language found; property verification recommended.</t>
+          <t>NOT FOUND / NEEDS CALL</t>
         </is>
       </c>
       <c r="AE9" s="2" t="inlineStr">
@@ -14099,35 +14083,33 @@
       </c>
       <c r="AQ9" s="2" t="inlineStr">
         <is>
-          <t>County multifamily inventory indicates family-focused property at same site as senior apartments. | Lake Panasoffkee Apartments - 352-793-2288</t>
+          <t>Lakeview Villas LTD | Clermont</t>
         </is>
       </c>
       <c r="AR9" s="2" t="n">
-        <v>87</v>
-      </c>
-      <c r="AS9" s="2" t="n">
-        <v>0</v>
-      </c>
+        <v>84</v>
+      </c>
+      <c r="AS9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Lakeview Villas LTD</t>
+          <t>Mirror Lake Manor</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>USDA RD</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>200 12th St Clermont</t>
+          <t>301 East Mirror Lk Fruitland Park</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Clermont</t>
+          <t>Fruitland Park</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -14143,7 +14125,7 @@
       <c r="G10" s="2" t="inlineStr"/>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>1 (352) 394-2896</t>
+          <t>1 352-728-4208</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr"/>
@@ -14153,7 +14135,7 @@
       <c r="M10" s="2" t="inlineStr"/>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://www.publichousing.com/city/fl-clermont</t>
+          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://www.publichousing.com/city/fl-fruitland_park</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
@@ -14161,25 +14143,21 @@
           <t>HUD/USDA/FHFC</t>
         </is>
       </c>
-      <c r="P10" s="2" t="inlineStr">
-        <is>
-          <t>1 bedroom</t>
-        </is>
-      </c>
+      <c r="P10" s="2" t="inlineStr"/>
       <c r="Q10" s="2" t="inlineStr"/>
       <c r="R10" s="2" t="inlineStr">
         <is>
-          <t>senior</t>
+          <t>disabled</t>
         </is>
       </c>
       <c r="S10" s="2" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>USDA RD 515</t>
         </is>
       </c>
       <c r="T10" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>income-based</t>
         </is>
       </c>
       <c r="U10" s="2" t="inlineStr">
@@ -14189,7 +14167,7 @@
       </c>
       <c r="V10" s="2" t="inlineStr">
         <is>
-          <t>NOT FOUND</t>
+          <t>Likely based on adjusted income; exact tenant rent requires application/property verification.</t>
         </is>
       </c>
       <c r="W10" s="2" t="inlineStr">
@@ -14282,33 +14260,35 @@
       </c>
       <c r="AQ10" s="2" t="inlineStr">
         <is>
-          <t>Lakeview Villas LTD | Clermont</t>
+          <t>Listed on USDA Rural Development Lake County property list. | Mirror Lake Manor | Fruitland Park Dr. | Mirror Lake Manor | Fruitland Park Dr. | Mirror Lake Manor | Fruitland Park Dr. | Mirror Lake Manor | Fruitland Park Dr. | Mirror Lake Manor | Fruitland Park Dr.</t>
         </is>
       </c>
       <c r="AR10" s="2" t="n">
         <v>84</v>
       </c>
-      <c r="AS10" s="2" t="inlineStr"/>
+      <c r="AS10" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Mirror Lake Manor</t>
+          <t>Pendry Villas</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>USDA RD</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>301 East Mirror Lk Fruitland Park</t>
+          <t>1303 2400 Kurt St</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Fruitland Park</t>
+          <t>Eustis</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -14324,7 +14304,7 @@
       <c r="G11" s="2" t="inlineStr"/>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>1 352-728-4208</t>
+          <t>(352) 357-3434</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr"/>
@@ -14334,7 +14314,7 @@
       <c r="M11" s="2" t="inlineStr"/>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://www.publichousing.com/city/fl-fruitland_park</t>
+          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://eustischamber.org/AboutEustis/housing.asp</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
@@ -14342,21 +14322,29 @@
           <t>HUD/USDA/FHFC</t>
         </is>
       </c>
-      <c r="P11" s="2" t="inlineStr"/>
-      <c r="Q11" s="2" t="inlineStr"/>
+      <c r="P11" s="2" t="inlineStr">
+        <is>
+          <t>4 bedroom, 4 bedrooms, 2 bedrooms, 3 bedrooms</t>
+        </is>
+      </c>
+      <c r="Q11" s="2" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
+      </c>
       <c r="R11" s="2" t="inlineStr">
         <is>
-          <t>disabled</t>
+          <t>senior</t>
         </is>
       </c>
       <c r="S11" s="2" t="inlineStr">
         <is>
-          <t>USDA RD 515</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="T11" s="2" t="inlineStr">
         <is>
-          <t>income-based</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="U11" s="2" t="inlineStr">
@@ -14366,7 +14354,7 @@
       </c>
       <c r="V11" s="2" t="inlineStr">
         <is>
-          <t>Likely based on adjusted income; exact tenant rent requires application/property verification.</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="W11" s="2" t="inlineStr">
@@ -14396,7 +14384,7 @@
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
-          <t>NOT FOUND / NEEDS CALL</t>
+          <t>Published pet-related language found; property verification recommended.</t>
         </is>
       </c>
       <c r="AC11" s="2" t="inlineStr">
@@ -14406,7 +14394,7 @@
       </c>
       <c r="AD11" s="2" t="inlineStr">
         <is>
-          <t>NOT FOUND / NEEDS CALL</t>
+          <t>Published credit-related language found; property verification recommended.</t>
         </is>
       </c>
       <c r="AE11" s="2" t="inlineStr">
@@ -14459,40 +14447,38 @@
       </c>
       <c r="AQ11" s="2" t="inlineStr">
         <is>
-          <t>Listed on USDA Rural Development Lake County property list. | Mirror Lake Manor | Fruitland Park Dr. | Mirror Lake Manor | Fruitland Park Dr. | Mirror Lake Manor | Fruitland Park Dr. | Mirror Lake Manor | Fruitland Park Dr. | Mirror Lake Manor | Fruitland Park Dr.</t>
+          <t>Pendry Villas | Eustis</t>
         </is>
       </c>
       <c r="AR11" s="2" t="n">
         <v>84</v>
       </c>
-      <c r="AS11" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="AS11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Pendry Villas</t>
+          <t>Panasoffkee Family Apartments</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Family</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>1303 2400 Kurt St</t>
+          <t>910 CR 482N</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Eustis</t>
+          <t>Lake Panasoffkee</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Lake County</t>
+          <t>Sumter County</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -14500,37 +14486,49 @@
           <t>FL</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr"/>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>33538</t>
+        </is>
+      </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>(352) 357-3434</t>
-        </is>
-      </c>
-      <c r="I12" s="2" t="inlineStr"/>
-      <c r="J12" s="2" t="inlineStr"/>
+          <t>(352) 793-2288</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>LowIncomeSupport@gmail.com</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>https://www.uslowcosthousing.com/foreclosure-housing/fl/lady_lake/fl-lady_lake-panasoffkee-family-apartments/</t>
+        </is>
+      </c>
       <c r="K12" s="2" t="inlineStr"/>
       <c r="L12" s="2" t="inlineStr"/>
-      <c r="M12" s="2" t="inlineStr"/>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>Sumter County Housing</t>
+        </is>
+      </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://eustischamber.org/AboutEustis/housing.asp</t>
+          <t>https://www.sumtercountyfl.gov/246/Rental-Assistance-Resources; https://www.sumtercountyfl.gov/DocumentCenter/View/29964/Sumter-County-Multifamily-Analysis-Final-Version-06202018; https://sumtercountyfl.gov/246/Rental-Assistance-Resources; https://www.lowincomehousing.us/FL/lake_panasoffkee.html; https://www.lowincomehousing.us/FL/sumterville.html; https://www.uslowcosthousing.com/foreclosure-housing/fl/lady_lake/fl-lady_lake-panasoffkee-family-apartments/; https://www.uslowcosthousing.com/foreclosure-housing/fl/sanford/fl-sanford-overlook-at-monroe-apartments/; https://www.lowincomehousing.us/FL/center_hill.html</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>HUD/USDA/FHFC</t>
+          <t>government</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>4 bedroom, 4 bedrooms, 2 bedrooms, 3 bedrooms</t>
-        </is>
-      </c>
-      <c r="Q12" s="2" t="inlineStr">
-        <is>
-          <t>47</t>
-        </is>
-      </c>
+          <t>1 bedroom, 2 bedroom, 3 bedroom</t>
+        </is>
+      </c>
+      <c r="Q12" s="2" t="inlineStr"/>
       <c r="R12" s="2" t="inlineStr">
         <is>
           <t>senior</t>
@@ -14538,12 +14536,12 @@
       </c>
       <c r="S12" s="2" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Unknown affordable rental</t>
         </is>
       </c>
       <c r="T12" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>income-based</t>
         </is>
       </c>
       <c r="U12" s="2" t="inlineStr">
@@ -14553,7 +14551,7 @@
       </c>
       <c r="V12" s="2" t="inlineStr">
         <is>
-          <t>NOT FOUND</t>
+          <t>Likely based on adjusted income; exact tenant rent requires application/property verification.</t>
         </is>
       </c>
       <c r="W12" s="2" t="inlineStr">
@@ -14583,7 +14581,7 @@
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
-          <t>Published pet-related language found; property verification recommended.</t>
+          <t>NOT FOUND / NEEDS CALL</t>
         </is>
       </c>
       <c r="AC12" s="2" t="inlineStr">
@@ -14646,13 +14644,15 @@
       </c>
       <c r="AQ12" s="2" t="inlineStr">
         <is>
-          <t>Pendry Villas | Eustis</t>
+          <t>County multifamily inventory indicates family-focused property at same site as senior apartments. | Lake Panasoffkee Apartments - 352-793-2288</t>
         </is>
       </c>
       <c r="AR12" s="2" t="n">
-        <v>84</v>
-      </c>
-      <c r="AS12" s="2" t="inlineStr"/>
+        <v>83</v>
+      </c>
+      <c r="AS12" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -16322,27 +16322,27 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Bushnell Garden Apartments</t>
+          <t>Fruitland Acres LTD</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>USDA RD</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>200 Jumper St S</t>
+          <t>303 Urick St</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Bushnell</t>
+          <t>Fruitland Park</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Sumter County</t>
+          <t>Lake County</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -16350,76 +16350,64 @@
           <t>FL</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr">
-        <is>
-          <t>33513</t>
-        </is>
-      </c>
+      <c r="G22" s="2" t="inlineStr"/>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>(352) 793-4838</t>
-        </is>
-      </c>
-      <c r="I22" s="2" t="inlineStr">
-        <is>
-          <t>LowIncomeSupport@gmail.com</t>
-        </is>
-      </c>
+          <t>(352) 323-3303</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr"/>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>https://affordablehousingonline.com/housing-search/Florida/Bushnell/Bushnell-Garden-Apartments/10000207</t>
+          <t>https://affordablehousingonline.com/housing-search/Florida/Fruitland-Park/Fruitland-Acres-Ltd/10026305</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>manges Bushnell Garden Apartments? Bushnell Garden Apartments is managed by Hale Management Group headquartered in Gainesville, Florida</t>
+          <t>private/corporate owners or nonprofits</t>
         </is>
       </c>
       <c r="L22" s="2" t="inlineStr"/>
-      <c r="M22" s="2" t="inlineStr">
-        <is>
-          <t>Sumter County Housing</t>
-        </is>
-      </c>
+      <c r="M22" s="2" t="inlineStr"/>
       <c r="N22" s="2" t="inlineStr">
         <is>
-          <t>https://www.sumtercountyfl.gov/246/Rental-Assistance-Resources; https://www.sumtercountyfl.gov/DocumentCenter/View/29964/Sumter-County-Multifamily-Analysis-Final-Version-06202018; https://sumtercountyfl.gov/246/Rental-Assistance-Resources; https://affordablehousingonline.com/housing-search/Florida/Bushnell/Bushnell-Garden-Apartments/10000207; https://www.lowincomehousing.us/FL/bushnell.html</t>
+          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://affordablehousingonline.com/housing-search/Florida/Fruitland-Park/Fruitland-Acres-Ltd/10026305; https://affordablehousingonline.com/housing-search/Florida/Fruitland-Park; https://affordablehousingonline.com/housing-search/Florida/Fruitland-Park/Mirror-Lake-Manor/10048622</t>
         </is>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>government</t>
+          <t>HUD/USDA/FHFC</t>
         </is>
       </c>
       <c r="P22" s="2" t="inlineStr">
         <is>
-          <t>3 Beds</t>
+          <t>2 Bed</t>
         </is>
       </c>
       <c r="Q22" s="2" t="inlineStr"/>
       <c r="R22" s="2" t="inlineStr">
         <is>
-          <t>senior</t>
+          <t>general low-income</t>
         </is>
       </c>
       <c r="S22" s="2" t="inlineStr">
         <is>
-          <t>Unknown affordable rental</t>
+          <t>USDA RD 515</t>
         </is>
       </c>
       <c r="T22" s="2" t="inlineStr">
         <is>
-          <t>fixed affordable rent</t>
+          <t>income-based</t>
         </is>
       </c>
       <c r="U22" s="2" t="inlineStr">
         <is>
-          <t>$600; $811; $700; $917; $775; $999</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="V22" s="2" t="inlineStr">
         <is>
-          <t>NOT FOUND</t>
+          <t>Likely based on adjusted income; exact tenant rent requires application/property verification.</t>
         </is>
       </c>
       <c r="W22" s="2" t="inlineStr">
@@ -16449,7 +16437,7 @@
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
-          <t>Published pet-related language found; property verification recommended.</t>
+          <t>NOT FOUND / NEEDS CALL</t>
         </is>
       </c>
       <c r="AC22" s="2" t="inlineStr">
@@ -16512,20 +16500,20 @@
       </c>
       <c r="AQ22" s="2" t="inlineStr">
         <is>
-          <t>Outside primary city list but near the target areas and listed by Sumter County as rental assistance provider. | Bushnell Garden Apartments - 352-793-4838</t>
+          <t>Listed on USDA Rural Development Lake County property list.</t>
         </is>
       </c>
       <c r="AR22" s="2" t="n">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="AS22" s="2" t="n">
-        <v>5.7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Fruitland Acres LTD</t>
+          <t>Montclair Village</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -16535,12 +16523,12 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>303 Urick St</t>
+          <t>2000 Park Cir</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Fruitland Park</t>
+          <t>Leesburg</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
@@ -16554,27 +16542,19 @@
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr"/>
-      <c r="H23" s="2" t="inlineStr">
-        <is>
-          <t>(352) 323-3303</t>
-        </is>
-      </c>
+      <c r="H23" s="2" t="inlineStr"/>
       <c r="I23" s="2" t="inlineStr"/>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>https://affordablehousingonline.com/housing-search/Florida/Fruitland-Park/Fruitland-Acres-Ltd/10026305</t>
-        </is>
-      </c>
-      <c r="K23" s="2" t="inlineStr">
-        <is>
-          <t>private/corporate owners or nonprofits</t>
-        </is>
-      </c>
+          <t>https://affordablehousingonline.com/housing-search/Florida/Leesburg/Montclair-Village/10103948</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr"/>
       <c r="L23" s="2" t="inlineStr"/>
       <c r="M23" s="2" t="inlineStr"/>
       <c r="N23" s="2" t="inlineStr">
         <is>
-          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://affordablehousingonline.com/housing-search/Florida/Fruitland-Park/Fruitland-Acres-Ltd/10026305; https://affordablehousingonline.com/housing-search/Florida/Fruitland-Park; https://affordablehousingonline.com/housing-search/Florida/Fruitland-Park/Mirror-Lake-Manor/10048622</t>
+          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://affordablehousingonline.com/housing-search/Florida/Leesburg/Montclair-Village/10103948; https://affordablehousingonline.com/housing-search/Florida/Leesburg</t>
         </is>
       </c>
       <c r="O23" s="2" t="inlineStr">
@@ -16590,7 +16570,7 @@
       <c r="Q23" s="2" t="inlineStr"/>
       <c r="R23" s="2" t="inlineStr">
         <is>
-          <t>general low-income</t>
+          <t>senior</t>
         </is>
       </c>
       <c r="S23" s="2" t="inlineStr">
@@ -16716,7 +16696,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Montclair Village</t>
+          <t>Palm Brook Apts LTD</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -16726,7 +16706,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>2000 Park Cir</t>
+          <t>37 Brook Cir</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -16749,15 +16729,19 @@
       <c r="I24" s="2" t="inlineStr"/>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>https://affordablehousingonline.com/housing-search/Florida/Leesburg/Montclair-Village/10103948</t>
-        </is>
-      </c>
-      <c r="K24" s="2" t="inlineStr"/>
+          <t>https://affordablehousingonline.com/housing-search/Florida/Leesburg/Palm-Brook-Apts-Ltd/10103487</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>private/corporate owners or nonprofits</t>
+        </is>
+      </c>
       <c r="L24" s="2" t="inlineStr"/>
       <c r="M24" s="2" t="inlineStr"/>
       <c r="N24" s="2" t="inlineStr">
         <is>
-          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://affordablehousingonline.com/housing-search/Florida/Leesburg/Montclair-Village/10103948; https://affordablehousingonline.com/housing-search/Florida/Leesburg</t>
+          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://affordablehousingonline.com/housing-search/Florida/Leesburg/Palm-Brook-Apts-Ltd/10103487; https://affordablehousingonline.com/housing-search/Florida/Leesburg</t>
         </is>
       </c>
       <c r="O24" s="2" t="inlineStr">
@@ -16899,7 +16883,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Palm Brook Apts LTD</t>
+          <t>Pepper Tree Apts</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -16909,7 +16893,7 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>37 Brook Cir</t>
+          <t>2503 South Street</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -16932,7 +16916,7 @@
       <c r="I25" s="2" t="inlineStr"/>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>https://affordablehousingonline.com/housing-search/Florida/Leesburg/Palm-Brook-Apts-Ltd/10103487</t>
+          <t>https://affordablehousingonline.com/housing-search/Florida/Leesburg/Pepper-Tree-Apts/10103485</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
@@ -16944,7 +16928,7 @@
       <c r="M25" s="2" t="inlineStr"/>
       <c r="N25" s="2" t="inlineStr">
         <is>
-          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://affordablehousingonline.com/housing-search/Florida/Leesburg/Palm-Brook-Apts-Ltd/10103487; https://affordablehousingonline.com/housing-search/Florida/Leesburg</t>
+          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://affordablehousingonline.com/housing-search/Florida/Leesburg/Pepper-Tree-Apts/10103485; https://affordablehousingonline.com/housing-search/Florida/Leesburg</t>
         </is>
       </c>
       <c r="O25" s="2" t="inlineStr">
@@ -17086,7 +17070,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Pepper Tree Apts</t>
+          <t>Pepper Tree Apts II</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -17119,7 +17103,7 @@
       <c r="I26" s="2" t="inlineStr"/>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>https://affordablehousingonline.com/housing-search/Florida/Leesburg/Pepper-Tree-Apts/10103485</t>
+          <t>https://affordablehousingonline.com/housing-search/Florida/Leesburg/Pepper-Tree-Apts-II/10104710</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr">
@@ -17131,7 +17115,7 @@
       <c r="M26" s="2" t="inlineStr"/>
       <c r="N26" s="2" t="inlineStr">
         <is>
-          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://affordablehousingonline.com/housing-search/Florida/Leesburg/Pepper-Tree-Apts/10103485; https://affordablehousingonline.com/housing-search/Florida/Leesburg</t>
+          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://affordablehousingonline.com/housing-search/Florida/Leesburg/Pepper-Tree-Apts-II/10104710; https://affordablehousingonline.com/housing-search/Florida/Leesburg</t>
         </is>
       </c>
       <c r="O26" s="2" t="inlineStr">
@@ -17273,27 +17257,27 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Pepper Tree Apts II</t>
+          <t>Bushnell Garden Apartments</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>USDA RD</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>2503 South Street</t>
+          <t>200 Jumper St S</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Leesburg</t>
+          <t>Bushnell</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Lake County</t>
+          <t>Sumter County</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
@@ -17301,34 +17285,50 @@
           <t>FL</t>
         </is>
       </c>
-      <c r="G27" s="2" t="inlineStr"/>
-      <c r="H27" s="2" t="inlineStr"/>
-      <c r="I27" s="2" t="inlineStr"/>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>33513</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>(352) 793-4838</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>LowIncomeSupport@gmail.com</t>
+        </is>
+      </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>https://affordablehousingonline.com/housing-search/Florida/Leesburg/Pepper-Tree-Apts-II/10104710</t>
+          <t>https://affordablehousingonline.com/housing-search/Florida/Bushnell/Bushnell-Garden-Apartments/10000207</t>
         </is>
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t>private/corporate owners or nonprofits</t>
+          <t>manges Bushnell Garden Apartments? Bushnell Garden Apartments is managed by Hale Management Group headquartered in Gainesville, Florida</t>
         </is>
       </c>
       <c r="L27" s="2" t="inlineStr"/>
-      <c r="M27" s="2" t="inlineStr"/>
+      <c r="M27" s="2" t="inlineStr">
+        <is>
+          <t>Sumter County Housing</t>
+        </is>
+      </c>
       <c r="N27" s="2" t="inlineStr">
         <is>
-          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://affordablehousingonline.com/housing-search/Florida/Leesburg/Pepper-Tree-Apts-II/10104710; https://affordablehousingonline.com/housing-search/Florida/Leesburg</t>
+          <t>https://www.sumtercountyfl.gov/246/Rental-Assistance-Resources; https://www.sumtercountyfl.gov/DocumentCenter/View/29964/Sumter-County-Multifamily-Analysis-Final-Version-06202018; https://sumtercountyfl.gov/246/Rental-Assistance-Resources; https://affordablehousingonline.com/housing-search/Florida/Bushnell/Bushnell-Garden-Apartments/10000207; https://www.lowincomehousing.us/FL/bushnell.html</t>
         </is>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t>HUD/USDA/FHFC</t>
+          <t>government</t>
         </is>
       </c>
       <c r="P27" s="2" t="inlineStr">
         <is>
-          <t>2 Bed</t>
+          <t>3 Beds</t>
         </is>
       </c>
       <c r="Q27" s="2" t="inlineStr"/>
@@ -17339,12 +17339,12 @@
       </c>
       <c r="S27" s="2" t="inlineStr">
         <is>
-          <t>USDA RD 515</t>
+          <t>Unknown affordable rental</t>
         </is>
       </c>
       <c r="T27" s="2" t="inlineStr">
         <is>
-          <t>income-based</t>
+          <t>fixed affordable rent</t>
         </is>
       </c>
       <c r="U27" s="2" t="inlineStr">
@@ -17354,7 +17354,7 @@
       </c>
       <c r="V27" s="2" t="inlineStr">
         <is>
-          <t>Likely based on adjusted income; exact tenant rent requires application/property verification.</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="W27" s="2" t="inlineStr">
@@ -17384,7 +17384,7 @@
       </c>
       <c r="AB27" s="2" t="inlineStr">
         <is>
-          <t>NOT FOUND / NEEDS CALL</t>
+          <t>Published pet-related language found; property verification recommended.</t>
         </is>
       </c>
       <c r="AC27" s="2" t="inlineStr">
@@ -17447,14 +17447,14 @@
       </c>
       <c r="AQ27" s="2" t="inlineStr">
         <is>
-          <t>Listed on USDA Rural Development Lake County property list.</t>
+          <t>Outside primary city list but near the target areas and listed by Sumter County as rental assistance provider. | Bushnell Garden Apartments - 352-793-4838</t>
         </is>
       </c>
       <c r="AR27" s="2" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AS27" s="2" t="n">
-        <v>0</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="28">
@@ -17532,12 +17532,12 @@
       </c>
       <c r="U28" s="2" t="inlineStr">
         <is>
-          <t>$911; $45,059; $152,928</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="V28" s="2" t="inlineStr">
         <is>
-          <t>NOT FOUND</t>
+          <t>Likely based on adjusted income; exact tenant rent requires application/property verification.</t>
         </is>
       </c>
       <c r="W28" s="2" t="inlineStr">
@@ -17638,7 +17638,7 @@
         </is>
       </c>
       <c r="AR28" s="2" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="AS28" s="2" t="n">
         <v>0</v>
@@ -17735,12 +17735,12 @@
       </c>
       <c r="U29" s="2" t="inlineStr">
         <is>
-          <t>$1558; $1638; $1857; $2362; $2849</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="V29" s="2" t="inlineStr">
         <is>
-          <t>Published amounts appear to be maximum restricted LIHTC rents; confirm actual tenant rent with property.</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="W29" s="2" t="inlineStr">
@@ -17841,7 +17841,7 @@
         </is>
       </c>
       <c r="AR29" s="2" t="n">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="AS29" s="2" t="inlineStr"/>
     </row>
@@ -18187,12 +18187,12 @@
       </c>
       <c r="U2" s="2" t="inlineStr">
         <is>
-          <t>$1558; $1638; $1857; $2362; $2849</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="V2" s="2" t="inlineStr">
         <is>
-          <t>Published amounts appear to be maximum restricted LIHTC rents; confirm actual tenant rent with property.</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="W2" s="2" t="inlineStr">
@@ -18293,7 +18293,7 @@
         </is>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>0</v>
@@ -18593,12 +18593,12 @@
       </c>
       <c r="U4" s="2" t="inlineStr">
         <is>
-          <t>$1558; $1638; $1857; $2362; $2849</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="V4" s="2" t="inlineStr">
         <is>
-          <t>Published amounts appear to be maximum restricted LIHTC rents; confirm actual tenant rent with property.</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="W4" s="2" t="inlineStr">
@@ -18699,7 +18699,7 @@
         </is>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>0</v>
@@ -18804,12 +18804,12 @@
       </c>
       <c r="U5" s="2" t="inlineStr">
         <is>
-          <t>$945; $951; $1250; $1572; $1665</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="V5" s="2" t="inlineStr">
         <is>
-          <t>Published amounts appear to be maximum restricted LIHTC rents; confirm actual tenant rent with property.</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="W5" s="2" t="inlineStr">
@@ -18910,7 +18910,7 @@
         </is>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>5.7</v>
@@ -18999,12 +18999,12 @@
       </c>
       <c r="U6" s="2" t="inlineStr">
         <is>
-          <t>$1558; $1638; $1857; $2362; $2849</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="V6" s="2" t="inlineStr">
         <is>
-          <t>Published amounts appear to be maximum restricted LIHTC rents; confirm actual tenant rent with property.</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="W6" s="2" t="inlineStr">
@@ -19105,7 +19105,7 @@
         </is>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="AS6" s="2" t="n">
         <v>0</v>
@@ -19210,12 +19210,12 @@
       </c>
       <c r="U7" s="2" t="inlineStr">
         <is>
-          <t>$945; $951; $1250; $1572; $1665</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="V7" s="2" t="inlineStr">
         <is>
-          <t>Published amounts appear to be maximum restricted LIHTC rents; confirm actual tenant rent with property.</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="W7" s="2" t="inlineStr">
@@ -19316,7 +19316,7 @@
         </is>
       </c>
       <c r="AR7" s="2" t="n">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="AS7" s="2" t="n">
         <v>0</v>
@@ -19413,12 +19413,12 @@
       </c>
       <c r="U8" s="2" t="inlineStr">
         <is>
-          <t>$1558; $1638; $18; $1857; $2362; $2849</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="V8" s="2" t="inlineStr">
         <is>
-          <t>Published amounts appear to be maximum restricted LIHTC rents; confirm actual tenant rent with property.</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="W8" s="2" t="inlineStr">
@@ -19519,34 +19519,34 @@
         </is>
       </c>
       <c r="AR8" s="2" t="n">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="AS8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Panasoffkee Family Apartments</t>
+          <t>Lakeview Villas LTD</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Family</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>910 CR 482N</t>
+          <t>200 12th St Clermont</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Lake Panasoffkee</t>
+          <t>Clermont</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Sumter County</t>
+          <t>Lake County</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -19554,46 +19554,30 @@
           <t>FL</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>33538</t>
-        </is>
-      </c>
+      <c r="G9" s="2" t="inlineStr"/>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>(352) 793-2288</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>LowIncomeSupport@gmail.com</t>
-        </is>
-      </c>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>https://www.uslowcosthousing.com/foreclosure-housing/fl/lady_lake/fl-lady_lake-panasoffkee-family-apartments/</t>
-        </is>
-      </c>
+          <t>1 (352) 394-2896</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr"/>
+      <c r="J9" s="2" t="inlineStr"/>
       <c r="K9" s="2" t="inlineStr"/>
       <c r="L9" s="2" t="inlineStr"/>
-      <c r="M9" s="2" t="inlineStr">
-        <is>
-          <t>Sumter County Housing</t>
-        </is>
-      </c>
+      <c r="M9" s="2" t="inlineStr"/>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>https://www.sumtercountyfl.gov/246/Rental-Assistance-Resources; https://www.sumtercountyfl.gov/DocumentCenter/View/29964/Sumter-County-Multifamily-Analysis-Final-Version-06202018; https://sumtercountyfl.gov/246/Rental-Assistance-Resources; https://www.lowincomehousing.us/FL/lake_panasoffkee.html; https://www.lowincomehousing.us/FL/sumterville.html; https://www.uslowcosthousing.com/foreclosure-housing/fl/lady_lake/fl-lady_lake-panasoffkee-family-apartments/; https://www.uslowcosthousing.com/foreclosure-housing/fl/sanford/fl-sanford-overlook-at-monroe-apartments/; https://www.lowincomehousing.us/FL/center_hill.html</t>
+          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://www.publichousing.com/city/fl-clermont</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>government</t>
+          <t>HUD/USDA/FHFC</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>1 bedroom, 2 bedroom, 3 bedroom</t>
+          <t>1 bedroom</t>
         </is>
       </c>
       <c r="Q9" s="2" t="inlineStr"/>
@@ -19604,17 +19588,17 @@
       </c>
       <c r="S9" s="2" t="inlineStr">
         <is>
-          <t>Unknown affordable rental</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="T9" s="2" t="inlineStr">
         <is>
-          <t>income-based</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="U9" s="2" t="inlineStr">
         <is>
-          <t>$48,400; $88,300; $59,500</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="V9" s="2" t="inlineStr">
@@ -19659,7 +19643,7 @@
       </c>
       <c r="AD9" s="2" t="inlineStr">
         <is>
-          <t>Published credit-related language found; property verification recommended.</t>
+          <t>NOT FOUND / NEEDS CALL</t>
         </is>
       </c>
       <c r="AE9" s="2" t="inlineStr">
@@ -19712,35 +19696,33 @@
       </c>
       <c r="AQ9" s="2" t="inlineStr">
         <is>
-          <t>County multifamily inventory indicates family-focused property at same site as senior apartments. | Lake Panasoffkee Apartments - 352-793-2288</t>
+          <t>Lakeview Villas LTD | Clermont</t>
         </is>
       </c>
       <c r="AR9" s="2" t="n">
-        <v>87</v>
-      </c>
-      <c r="AS9" s="2" t="n">
-        <v>0</v>
-      </c>
+        <v>84</v>
+      </c>
+      <c r="AS9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Lakeview Villas LTD</t>
+          <t>Mirror Lake Manor</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>USDA RD</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>200 12th St Clermont</t>
+          <t>301 East Mirror Lk Fruitland Park</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Clermont</t>
+          <t>Fruitland Park</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -19756,7 +19738,7 @@
       <c r="G10" s="2" t="inlineStr"/>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>1 (352) 394-2896</t>
+          <t>1 352-728-4208</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr"/>
@@ -19766,7 +19748,7 @@
       <c r="M10" s="2" t="inlineStr"/>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://www.publichousing.com/city/fl-clermont</t>
+          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://www.publichousing.com/city/fl-fruitland_park</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
@@ -19774,25 +19756,21 @@
           <t>HUD/USDA/FHFC</t>
         </is>
       </c>
-      <c r="P10" s="2" t="inlineStr">
-        <is>
-          <t>1 bedroom</t>
-        </is>
-      </c>
+      <c r="P10" s="2" t="inlineStr"/>
       <c r="Q10" s="2" t="inlineStr"/>
       <c r="R10" s="2" t="inlineStr">
         <is>
-          <t>senior</t>
+          <t>disabled</t>
         </is>
       </c>
       <c r="S10" s="2" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>USDA RD 515</t>
         </is>
       </c>
       <c r="T10" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>income-based</t>
         </is>
       </c>
       <c r="U10" s="2" t="inlineStr">
@@ -19802,7 +19780,7 @@
       </c>
       <c r="V10" s="2" t="inlineStr">
         <is>
-          <t>NOT FOUND</t>
+          <t>Likely based on adjusted income; exact tenant rent requires application/property verification.</t>
         </is>
       </c>
       <c r="W10" s="2" t="inlineStr">
@@ -19895,33 +19873,35 @@
       </c>
       <c r="AQ10" s="2" t="inlineStr">
         <is>
-          <t>Lakeview Villas LTD | Clermont</t>
+          <t>Listed on USDA Rural Development Lake County property list. | Mirror Lake Manor | Fruitland Park Dr. | Mirror Lake Manor | Fruitland Park Dr. | Mirror Lake Manor | Fruitland Park Dr. | Mirror Lake Manor | Fruitland Park Dr. | Mirror Lake Manor | Fruitland Park Dr.</t>
         </is>
       </c>
       <c r="AR10" s="2" t="n">
         <v>84</v>
       </c>
-      <c r="AS10" s="2" t="inlineStr"/>
+      <c r="AS10" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Mirror Lake Manor</t>
+          <t>Pendry Villas</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>USDA RD</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>301 East Mirror Lk Fruitland Park</t>
+          <t>1303 2400 Kurt St</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Fruitland Park</t>
+          <t>Eustis</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -19937,7 +19917,7 @@
       <c r="G11" s="2" t="inlineStr"/>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>1 352-728-4208</t>
+          <t>(352) 357-3434</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr"/>
@@ -19947,7 +19927,7 @@
       <c r="M11" s="2" t="inlineStr"/>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://www.publichousing.com/city/fl-fruitland_park</t>
+          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://eustischamber.org/AboutEustis/housing.asp</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
@@ -19955,21 +19935,29 @@
           <t>HUD/USDA/FHFC</t>
         </is>
       </c>
-      <c r="P11" s="2" t="inlineStr"/>
-      <c r="Q11" s="2" t="inlineStr"/>
+      <c r="P11" s="2" t="inlineStr">
+        <is>
+          <t>4 bedroom, 4 bedrooms, 2 bedrooms, 3 bedrooms</t>
+        </is>
+      </c>
+      <c r="Q11" s="2" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
+      </c>
       <c r="R11" s="2" t="inlineStr">
         <is>
-          <t>disabled</t>
+          <t>senior</t>
         </is>
       </c>
       <c r="S11" s="2" t="inlineStr">
         <is>
-          <t>USDA RD 515</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="T11" s="2" t="inlineStr">
         <is>
-          <t>income-based</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="U11" s="2" t="inlineStr">
@@ -19979,7 +19967,7 @@
       </c>
       <c r="V11" s="2" t="inlineStr">
         <is>
-          <t>Likely based on adjusted income; exact tenant rent requires application/property verification.</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="W11" s="2" t="inlineStr">
@@ -20009,7 +19997,7 @@
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
-          <t>NOT FOUND / NEEDS CALL</t>
+          <t>Published pet-related language found; property verification recommended.</t>
         </is>
       </c>
       <c r="AC11" s="2" t="inlineStr">
@@ -20019,7 +20007,7 @@
       </c>
       <c r="AD11" s="2" t="inlineStr">
         <is>
-          <t>NOT FOUND / NEEDS CALL</t>
+          <t>Published credit-related language found; property verification recommended.</t>
         </is>
       </c>
       <c r="AE11" s="2" t="inlineStr">
@@ -20072,40 +20060,38 @@
       </c>
       <c r="AQ11" s="2" t="inlineStr">
         <is>
-          <t>Listed on USDA Rural Development Lake County property list. | Mirror Lake Manor | Fruitland Park Dr. | Mirror Lake Manor | Fruitland Park Dr. | Mirror Lake Manor | Fruitland Park Dr. | Mirror Lake Manor | Fruitland Park Dr. | Mirror Lake Manor | Fruitland Park Dr.</t>
+          <t>Pendry Villas | Eustis</t>
         </is>
       </c>
       <c r="AR11" s="2" t="n">
         <v>84</v>
       </c>
-      <c r="AS11" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="AS11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Pendry Villas</t>
+          <t>Panasoffkee Family Apartments</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Family</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>1303 2400 Kurt St</t>
+          <t>910 CR 482N</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Eustis</t>
+          <t>Lake Panasoffkee</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Lake County</t>
+          <t>Sumter County</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -20113,37 +20099,49 @@
           <t>FL</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr"/>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>33538</t>
+        </is>
+      </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>(352) 357-3434</t>
-        </is>
-      </c>
-      <c r="I12" s="2" t="inlineStr"/>
-      <c r="J12" s="2" t="inlineStr"/>
+          <t>(352) 793-2288</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>LowIncomeSupport@gmail.com</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>https://www.uslowcosthousing.com/foreclosure-housing/fl/lady_lake/fl-lady_lake-panasoffkee-family-apartments/</t>
+        </is>
+      </c>
       <c r="K12" s="2" t="inlineStr"/>
       <c r="L12" s="2" t="inlineStr"/>
-      <c r="M12" s="2" t="inlineStr"/>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>Sumter County Housing</t>
+        </is>
+      </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://eustischamber.org/AboutEustis/housing.asp</t>
+          <t>https://www.sumtercountyfl.gov/246/Rental-Assistance-Resources; https://www.sumtercountyfl.gov/DocumentCenter/View/29964/Sumter-County-Multifamily-Analysis-Final-Version-06202018; https://sumtercountyfl.gov/246/Rental-Assistance-Resources; https://www.lowincomehousing.us/FL/lake_panasoffkee.html; https://www.lowincomehousing.us/FL/sumterville.html; https://www.uslowcosthousing.com/foreclosure-housing/fl/lady_lake/fl-lady_lake-panasoffkee-family-apartments/; https://www.uslowcosthousing.com/foreclosure-housing/fl/sanford/fl-sanford-overlook-at-monroe-apartments/; https://www.lowincomehousing.us/FL/center_hill.html</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>HUD/USDA/FHFC</t>
+          <t>government</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>4 bedroom, 4 bedrooms, 2 bedrooms, 3 bedrooms</t>
-        </is>
-      </c>
-      <c r="Q12" s="2" t="inlineStr">
-        <is>
-          <t>47</t>
-        </is>
-      </c>
+          <t>1 bedroom, 2 bedroom, 3 bedroom</t>
+        </is>
+      </c>
+      <c r="Q12" s="2" t="inlineStr"/>
       <c r="R12" s="2" t="inlineStr">
         <is>
           <t>senior</t>
@@ -20151,12 +20149,12 @@
       </c>
       <c r="S12" s="2" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Unknown affordable rental</t>
         </is>
       </c>
       <c r="T12" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>income-based</t>
         </is>
       </c>
       <c r="U12" s="2" t="inlineStr">
@@ -20166,7 +20164,7 @@
       </c>
       <c r="V12" s="2" t="inlineStr">
         <is>
-          <t>NOT FOUND</t>
+          <t>Likely based on adjusted income; exact tenant rent requires application/property verification.</t>
         </is>
       </c>
       <c r="W12" s="2" t="inlineStr">
@@ -20196,7 +20194,7 @@
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
-          <t>Published pet-related language found; property verification recommended.</t>
+          <t>NOT FOUND / NEEDS CALL</t>
         </is>
       </c>
       <c r="AC12" s="2" t="inlineStr">
@@ -20259,13 +20257,15 @@
       </c>
       <c r="AQ12" s="2" t="inlineStr">
         <is>
-          <t>Pendry Villas | Eustis</t>
+          <t>County multifamily inventory indicates family-focused property at same site as senior apartments. | Lake Panasoffkee Apartments - 352-793-2288</t>
         </is>
       </c>
       <c r="AR12" s="2" t="n">
-        <v>84</v>
-      </c>
-      <c r="AS12" s="2" t="inlineStr"/>
+        <v>83</v>
+      </c>
+      <c r="AS12" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -21740,27 +21740,27 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Bushnell Garden Apartments</t>
+          <t>Fruitland Acres LTD</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>USDA RD</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>200 Jumper St S</t>
+          <t>303 Urick St</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Bushnell</t>
+          <t>Fruitland Park</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Sumter County</t>
+          <t>Lake County</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
@@ -21768,76 +21768,64 @@
           <t>FL</t>
         </is>
       </c>
-      <c r="G21" s="2" t="inlineStr">
-        <is>
-          <t>33513</t>
-        </is>
-      </c>
+      <c r="G21" s="2" t="inlineStr"/>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>(352) 793-4838</t>
-        </is>
-      </c>
-      <c r="I21" s="2" t="inlineStr">
-        <is>
-          <t>LowIncomeSupport@gmail.com</t>
-        </is>
-      </c>
+          <t>(352) 323-3303</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr"/>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>https://affordablehousingonline.com/housing-search/Florida/Bushnell/Bushnell-Garden-Apartments/10000207</t>
+          <t>https://affordablehousingonline.com/housing-search/Florida/Fruitland-Park/Fruitland-Acres-Ltd/10026305</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>manges Bushnell Garden Apartments? Bushnell Garden Apartments is managed by Hale Management Group headquartered in Gainesville, Florida</t>
+          <t>private/corporate owners or nonprofits</t>
         </is>
       </c>
       <c r="L21" s="2" t="inlineStr"/>
-      <c r="M21" s="2" t="inlineStr">
-        <is>
-          <t>Sumter County Housing</t>
-        </is>
-      </c>
+      <c r="M21" s="2" t="inlineStr"/>
       <c r="N21" s="2" t="inlineStr">
         <is>
-          <t>https://www.sumtercountyfl.gov/246/Rental-Assistance-Resources; https://www.sumtercountyfl.gov/DocumentCenter/View/29964/Sumter-County-Multifamily-Analysis-Final-Version-06202018; https://sumtercountyfl.gov/246/Rental-Assistance-Resources; https://affordablehousingonline.com/housing-search/Florida/Bushnell/Bushnell-Garden-Apartments/10000207; https://www.lowincomehousing.us/FL/bushnell.html</t>
+          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://affordablehousingonline.com/housing-search/Florida/Fruitland-Park/Fruitland-Acres-Ltd/10026305; https://affordablehousingonline.com/housing-search/Florida/Fruitland-Park; https://affordablehousingonline.com/housing-search/Florida/Fruitland-Park/Mirror-Lake-Manor/10048622</t>
         </is>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>government</t>
+          <t>HUD/USDA/FHFC</t>
         </is>
       </c>
       <c r="P21" s="2" t="inlineStr">
         <is>
-          <t>3 Beds</t>
+          <t>2 Bed</t>
         </is>
       </c>
       <c r="Q21" s="2" t="inlineStr"/>
       <c r="R21" s="2" t="inlineStr">
         <is>
-          <t>senior</t>
+          <t>general low-income</t>
         </is>
       </c>
       <c r="S21" s="2" t="inlineStr">
         <is>
-          <t>Unknown affordable rental</t>
+          <t>USDA RD 515</t>
         </is>
       </c>
       <c r="T21" s="2" t="inlineStr">
         <is>
-          <t>fixed affordable rent</t>
+          <t>income-based</t>
         </is>
       </c>
       <c r="U21" s="2" t="inlineStr">
         <is>
-          <t>$600; $811; $700; $917; $775; $999</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="V21" s="2" t="inlineStr">
         <is>
-          <t>NOT FOUND</t>
+          <t>Likely based on adjusted income; exact tenant rent requires application/property verification.</t>
         </is>
       </c>
       <c r="W21" s="2" t="inlineStr">
@@ -21867,7 +21855,7 @@
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
-          <t>Published pet-related language found; property verification recommended.</t>
+          <t>NOT FOUND / NEEDS CALL</t>
         </is>
       </c>
       <c r="AC21" s="2" t="inlineStr">
@@ -21930,20 +21918,20 @@
       </c>
       <c r="AQ21" s="2" t="inlineStr">
         <is>
-          <t>Outside primary city list but near the target areas and listed by Sumter County as rental assistance provider. | Bushnell Garden Apartments - 352-793-4838</t>
+          <t>Listed on USDA Rural Development Lake County property list.</t>
         </is>
       </c>
       <c r="AR21" s="2" t="n">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="AS21" s="2" t="n">
-        <v>5.7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Fruitland Acres LTD</t>
+          <t>Montclair Village</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -21953,12 +21941,12 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>303 Urick St</t>
+          <t>2000 Park Cir</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Fruitland Park</t>
+          <t>Leesburg</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -21972,27 +21960,19 @@
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr"/>
-      <c r="H22" s="2" t="inlineStr">
-        <is>
-          <t>(352) 323-3303</t>
-        </is>
-      </c>
+      <c r="H22" s="2" t="inlineStr"/>
       <c r="I22" s="2" t="inlineStr"/>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>https://affordablehousingonline.com/housing-search/Florida/Fruitland-Park/Fruitland-Acres-Ltd/10026305</t>
-        </is>
-      </c>
-      <c r="K22" s="2" t="inlineStr">
-        <is>
-          <t>private/corporate owners or nonprofits</t>
-        </is>
-      </c>
+          <t>https://affordablehousingonline.com/housing-search/Florida/Leesburg/Montclair-Village/10103948</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr"/>
       <c r="L22" s="2" t="inlineStr"/>
       <c r="M22" s="2" t="inlineStr"/>
       <c r="N22" s="2" t="inlineStr">
         <is>
-          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://affordablehousingonline.com/housing-search/Florida/Fruitland-Park/Fruitland-Acres-Ltd/10026305; https://affordablehousingonline.com/housing-search/Florida/Fruitland-Park; https://affordablehousingonline.com/housing-search/Florida/Fruitland-Park/Mirror-Lake-Manor/10048622</t>
+          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://affordablehousingonline.com/housing-search/Florida/Leesburg/Montclair-Village/10103948; https://affordablehousingonline.com/housing-search/Florida/Leesburg</t>
         </is>
       </c>
       <c r="O22" s="2" t="inlineStr">
@@ -22008,7 +21988,7 @@
       <c r="Q22" s="2" t="inlineStr"/>
       <c r="R22" s="2" t="inlineStr">
         <is>
-          <t>general low-income</t>
+          <t>senior</t>
         </is>
       </c>
       <c r="S22" s="2" t="inlineStr">
@@ -22134,7 +22114,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Montclair Village</t>
+          <t>Palm Brook Apts LTD</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -22144,7 +22124,7 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>2000 Park Cir</t>
+          <t>37 Brook Cir</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -22167,15 +22147,19 @@
       <c r="I23" s="2" t="inlineStr"/>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>https://affordablehousingonline.com/housing-search/Florida/Leesburg/Montclair-Village/10103948</t>
-        </is>
-      </c>
-      <c r="K23" s="2" t="inlineStr"/>
+          <t>https://affordablehousingonline.com/housing-search/Florida/Leesburg/Palm-Brook-Apts-Ltd/10103487</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>private/corporate owners or nonprofits</t>
+        </is>
+      </c>
       <c r="L23" s="2" t="inlineStr"/>
       <c r="M23" s="2" t="inlineStr"/>
       <c r="N23" s="2" t="inlineStr">
         <is>
-          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://affordablehousingonline.com/housing-search/Florida/Leesburg/Montclair-Village/10103948; https://affordablehousingonline.com/housing-search/Florida/Leesburg</t>
+          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://affordablehousingonline.com/housing-search/Florida/Leesburg/Palm-Brook-Apts-Ltd/10103487; https://affordablehousingonline.com/housing-search/Florida/Leesburg</t>
         </is>
       </c>
       <c r="O23" s="2" t="inlineStr">
@@ -22317,7 +22301,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Palm Brook Apts LTD</t>
+          <t>Pepper Tree Apts</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -22327,7 +22311,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>37 Brook Cir</t>
+          <t>2503 South Street</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -22350,7 +22334,7 @@
       <c r="I24" s="2" t="inlineStr"/>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>https://affordablehousingonline.com/housing-search/Florida/Leesburg/Palm-Brook-Apts-Ltd/10103487</t>
+          <t>https://affordablehousingonline.com/housing-search/Florida/Leesburg/Pepper-Tree-Apts/10103485</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
@@ -22362,7 +22346,7 @@
       <c r="M24" s="2" t="inlineStr"/>
       <c r="N24" s="2" t="inlineStr">
         <is>
-          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://affordablehousingonline.com/housing-search/Florida/Leesburg/Palm-Brook-Apts-Ltd/10103487; https://affordablehousingonline.com/housing-search/Florida/Leesburg</t>
+          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://affordablehousingonline.com/housing-search/Florida/Leesburg/Pepper-Tree-Apts/10103485; https://affordablehousingonline.com/housing-search/Florida/Leesburg</t>
         </is>
       </c>
       <c r="O24" s="2" t="inlineStr">
@@ -22504,7 +22488,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Pepper Tree Apts</t>
+          <t>Pepper Tree Apts II</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -22537,7 +22521,7 @@
       <c r="I25" s="2" t="inlineStr"/>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>https://affordablehousingonline.com/housing-search/Florida/Leesburg/Pepper-Tree-Apts/10103485</t>
+          <t>https://affordablehousingonline.com/housing-search/Florida/Leesburg/Pepper-Tree-Apts-II/10104710</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
@@ -22549,7 +22533,7 @@
       <c r="M25" s="2" t="inlineStr"/>
       <c r="N25" s="2" t="inlineStr">
         <is>
-          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://affordablehousingonline.com/housing-search/Florida/Leesburg/Pepper-Tree-Apts/10103485; https://affordablehousingonline.com/housing-search/Florida/Leesburg</t>
+          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://affordablehousingonline.com/housing-search/Florida/Leesburg/Pepper-Tree-Apts-II/10104710; https://affordablehousingonline.com/housing-search/Florida/Leesburg</t>
         </is>
       </c>
       <c r="O25" s="2" t="inlineStr">
@@ -22691,27 +22675,27 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Pepper Tree Apts II</t>
+          <t>Bushnell Garden Apartments</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>USDA RD</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>2503 South Street</t>
+          <t>200 Jumper St S</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Leesburg</t>
+          <t>Bushnell</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Lake County</t>
+          <t>Sumter County</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -22719,34 +22703,50 @@
           <t>FL</t>
         </is>
       </c>
-      <c r="G26" s="2" t="inlineStr"/>
-      <c r="H26" s="2" t="inlineStr"/>
-      <c r="I26" s="2" t="inlineStr"/>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>33513</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>(352) 793-4838</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>LowIncomeSupport@gmail.com</t>
+        </is>
+      </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>https://affordablehousingonline.com/housing-search/Florida/Leesburg/Pepper-Tree-Apts-II/10104710</t>
+          <t>https://affordablehousingonline.com/housing-search/Florida/Bushnell/Bushnell-Garden-Apartments/10000207</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t>private/corporate owners or nonprofits</t>
+          <t>manges Bushnell Garden Apartments? Bushnell Garden Apartments is managed by Hale Management Group headquartered in Gainesville, Florida</t>
         </is>
       </c>
       <c r="L26" s="2" t="inlineStr"/>
-      <c r="M26" s="2" t="inlineStr"/>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>Sumter County Housing</t>
+        </is>
+      </c>
       <c r="N26" s="2" t="inlineStr">
         <is>
-          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://affordablehousingonline.com/housing-search/Florida/Leesburg/Pepper-Tree-Apts-II/10104710; https://affordablehousingonline.com/housing-search/Florida/Leesburg</t>
+          <t>https://www.sumtercountyfl.gov/246/Rental-Assistance-Resources; https://www.sumtercountyfl.gov/DocumentCenter/View/29964/Sumter-County-Multifamily-Analysis-Final-Version-06202018; https://sumtercountyfl.gov/246/Rental-Assistance-Resources; https://affordablehousingonline.com/housing-search/Florida/Bushnell/Bushnell-Garden-Apartments/10000207; https://www.lowincomehousing.us/FL/bushnell.html</t>
         </is>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
-          <t>HUD/USDA/FHFC</t>
+          <t>government</t>
         </is>
       </c>
       <c r="P26" s="2" t="inlineStr">
         <is>
-          <t>2 Bed</t>
+          <t>3 Beds</t>
         </is>
       </c>
       <c r="Q26" s="2" t="inlineStr"/>
@@ -22757,12 +22757,12 @@
       </c>
       <c r="S26" s="2" t="inlineStr">
         <is>
-          <t>USDA RD 515</t>
+          <t>Unknown affordable rental</t>
         </is>
       </c>
       <c r="T26" s="2" t="inlineStr">
         <is>
-          <t>income-based</t>
+          <t>fixed affordable rent</t>
         </is>
       </c>
       <c r="U26" s="2" t="inlineStr">
@@ -22772,7 +22772,7 @@
       </c>
       <c r="V26" s="2" t="inlineStr">
         <is>
-          <t>Likely based on adjusted income; exact tenant rent requires application/property verification.</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="W26" s="2" t="inlineStr">
@@ -22802,7 +22802,7 @@
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
-          <t>NOT FOUND / NEEDS CALL</t>
+          <t>Published pet-related language found; property verification recommended.</t>
         </is>
       </c>
       <c r="AC26" s="2" t="inlineStr">
@@ -22865,14 +22865,14 @@
       </c>
       <c r="AQ26" s="2" t="inlineStr">
         <is>
-          <t>Listed on USDA Rural Development Lake County property list.</t>
+          <t>Outside primary city list but near the target areas and listed by Sumter County as rental assistance provider. | Bushnell Garden Apartments - 352-793-4838</t>
         </is>
       </c>
       <c r="AR26" s="2" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AS26" s="2" t="n">
-        <v>0</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="27">
@@ -22966,12 +22966,12 @@
       </c>
       <c r="U27" s="2" t="inlineStr">
         <is>
-          <t>$1558; $1638; $1857; $2362; $2849</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="V27" s="2" t="inlineStr">
         <is>
-          <t>Published amounts appear to be maximum restricted LIHTC rents; confirm actual tenant rent with property.</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
       <c r="W27" s="2" t="inlineStr">
@@ -23072,7 +23072,7 @@
         </is>
       </c>
       <c r="AR27" s="2" t="n">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="AS27" s="2" t="inlineStr"/>
     </row>
@@ -23371,12 +23371,12 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Panasoffkee Family Apartments</t>
+          <t>Lakeview Villas LTD</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>(352) 793-2288</t>
+          <t>1 (352) 394-2896</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -23404,12 +23404,12 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Lakeview Villas LTD</t>
+          <t>Mirror Lake Manor</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>1 (352) 394-2896</t>
+          <t>1 352-728-4208</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -23437,12 +23437,12 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Mirror Lake Manor</t>
+          <t>Pendry Villas</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>1 352-728-4208</t>
+          <t>(352) 357-3434</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -23470,12 +23470,12 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Pendry Villas</t>
+          <t>Panasoffkee Family Apartments</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>(352) 357-3434</t>
+          <t>(352) 793-2288</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -23792,12 +23792,12 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Bushnell Garden Apartments</t>
+          <t>Fruitland Acres LTD</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>(352) 793-4838</t>
+          <t>(352) 323-3303</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -23825,14 +23825,10 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Fruitland Acres LTD</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>(352) 323-3303</t>
-        </is>
-      </c>
+          <t>Montclair Village</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr"/>
       <c r="C23" s="2" t="inlineStr">
         <is>
           <t>NOT FOUND / NEEDS CALL</t>
@@ -23858,7 +23854,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Montclair Village</t>
+          <t>Palm Brook Apts LTD</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr"/>
@@ -23887,7 +23883,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Palm Brook Apts LTD</t>
+          <t>Pepper Tree Apts</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr"/>
@@ -23916,7 +23912,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Pepper Tree Apts</t>
+          <t>Pepper Tree Apts II</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr"/>
@@ -23945,10 +23941,14 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Pepper Tree Apts II</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr"/>
+          <t>Bushnell Garden Apartments</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>(352) 793-4838</t>
+        </is>
+      </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
           <t>NOT FOUND / NEEDS CALL</t>
@@ -24231,12 +24231,12 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Panasoffkee Family Apartments</t>
+          <t>Lakeview Villas LTD</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>https://www.sumtercountyfl.gov/246/Rental-Assistance-Resources; https://www.sumtercountyfl.gov/DocumentCenter/View/29964/Sumter-County-Multifamily-Analysis-Final-Version-06202018; https://sumtercountyfl.gov/246/Rental-Assistance-Resources; https://www.lowincomehousing.us/FL/lake_panasoffkee.html; https://www.lowincomehousing.us/FL/sumterville.html; https://www.uslowcosthousing.com/foreclosure-housing/fl/lady_lake/fl-lady_lake-panasoffkee-family-apartments/; https://www.uslowcosthousing.com/foreclosure-housing/fl/sanford/fl-sanford-overlook-at-monroe-apartments/; https://www.lowincomehousing.us/FL/center_hill.html</t>
+          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://www.publichousing.com/city/fl-clermont</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -24246,19 +24246,19 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>County multifamily inventory indicates family-focused property at same site as senior apartments. | Lake Panasoffkee Apartments - 352-793-2288</t>
+          <t>Lakeview Villas LTD | Clermont</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Lakeview Villas LTD</t>
+          <t>Mirror Lake Manor</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://www.publichousing.com/city/fl-clermont</t>
+          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://www.publichousing.com/city/fl-fruitland_park</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -24268,19 +24268,19 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Lakeview Villas LTD | Clermont</t>
+          <t>Listed on USDA Rural Development Lake County property list. | Mirror Lake Manor | Fruitland Park Dr. | Mirror Lake Manor | Fruitland Park Dr. | Mirror Lake Manor | Fruitland Park Dr. | Mirror Lake Manor | Fruitland Park Dr. | Mirror Lake Manor | Fruitland Park Dr.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Mirror Lake Manor</t>
+          <t>Pendry Villas</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://www.publichousing.com/city/fl-fruitland_park</t>
+          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://eustischamber.org/AboutEustis/housing.asp</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -24290,19 +24290,19 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Listed on USDA Rural Development Lake County property list. | Mirror Lake Manor | Fruitland Park Dr. | Mirror Lake Manor | Fruitland Park Dr. | Mirror Lake Manor | Fruitland Park Dr. | Mirror Lake Manor | Fruitland Park Dr. | Mirror Lake Manor | Fruitland Park Dr.</t>
+          <t>Pendry Villas | Eustis</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Pendry Villas</t>
+          <t>Panasoffkee Family Apartments</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://eustischamber.org/AboutEustis/housing.asp</t>
+          <t>https://www.sumtercountyfl.gov/246/Rental-Assistance-Resources; https://www.sumtercountyfl.gov/DocumentCenter/View/29964/Sumter-County-Multifamily-Analysis-Final-Version-06202018; https://sumtercountyfl.gov/246/Rental-Assistance-Resources; https://www.lowincomehousing.us/FL/lake_panasoffkee.html; https://www.lowincomehousing.us/FL/sumterville.html; https://www.uslowcosthousing.com/foreclosure-housing/fl/lady_lake/fl-lady_lake-panasoffkee-family-apartments/; https://www.uslowcosthousing.com/foreclosure-housing/fl/sanford/fl-sanford-overlook-at-monroe-apartments/; https://www.lowincomehousing.us/FL/center_hill.html</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -24312,7 +24312,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Pendry Villas | Eustis</t>
+          <t>County multifamily inventory indicates family-focused property at same site as senior apartments. | Lake Panasoffkee Apartments - 352-793-2288</t>
         </is>
       </c>
     </row>
@@ -24517,12 +24517,12 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Bushnell Garden Apartments</t>
+          <t>Fruitland Acres LTD</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>https://www.sumtercountyfl.gov/246/Rental-Assistance-Resources; https://www.sumtercountyfl.gov/DocumentCenter/View/29964/Sumter-County-Multifamily-Analysis-Final-Version-06202018; https://sumtercountyfl.gov/246/Rental-Assistance-Resources; https://affordablehousingonline.com/housing-search/Florida/Bushnell/Bushnell-Garden-Apartments/10000207; https://www.lowincomehousing.us/FL/bushnell.html</t>
+          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://affordablehousingonline.com/housing-search/Florida/Fruitland-Park/Fruitland-Acres-Ltd/10026305; https://affordablehousingonline.com/housing-search/Florida/Fruitland-Park; https://affordablehousingonline.com/housing-search/Florida/Fruitland-Park/Mirror-Lake-Manor/10048622</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -24532,19 +24532,19 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Outside primary city list but near the target areas and listed by Sumter County as rental assistance provider. | Bushnell Garden Apartments - 352-793-4838</t>
+          <t>Listed on USDA Rural Development Lake County property list.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Fruitland Acres LTD</t>
+          <t>Montclair Village</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://affordablehousingonline.com/housing-search/Florida/Fruitland-Park/Fruitland-Acres-Ltd/10026305; https://affordablehousingonline.com/housing-search/Florida/Fruitland-Park; https://affordablehousingonline.com/housing-search/Florida/Fruitland-Park/Mirror-Lake-Manor/10048622</t>
+          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://affordablehousingonline.com/housing-search/Florida/Leesburg/Montclair-Village/10103948; https://affordablehousingonline.com/housing-search/Florida/Leesburg</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -24561,12 +24561,12 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Montclair Village</t>
+          <t>Palm Brook Apts LTD</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://affordablehousingonline.com/housing-search/Florida/Leesburg/Montclair-Village/10103948; https://affordablehousingonline.com/housing-search/Florida/Leesburg</t>
+          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://affordablehousingonline.com/housing-search/Florida/Leesburg/Palm-Brook-Apts-Ltd/10103487; https://affordablehousingonline.com/housing-search/Florida/Leesburg</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -24583,12 +24583,12 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Palm Brook Apts LTD</t>
+          <t>Pepper Tree Apts</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://affordablehousingonline.com/housing-search/Florida/Leesburg/Palm-Brook-Apts-Ltd/10103487; https://affordablehousingonline.com/housing-search/Florida/Leesburg</t>
+          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://affordablehousingonline.com/housing-search/Florida/Leesburg/Pepper-Tree-Apts/10103485; https://affordablehousingonline.com/housing-search/Florida/Leesburg</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -24605,12 +24605,12 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Pepper Tree Apts</t>
+          <t>Pepper Tree Apts II</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://affordablehousingonline.com/housing-search/Florida/Leesburg/Pepper-Tree-Apts/10103485; https://affordablehousingonline.com/housing-search/Florida/Leesburg</t>
+          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://affordablehousingonline.com/housing-search/Florida/Leesburg/Pepper-Tree-Apts-II/10104710; https://affordablehousingonline.com/housing-search/Florida/Leesburg</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -24627,12 +24627,12 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Pepper Tree Apts II</t>
+          <t>Bushnell Garden Apartments</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>https://rdmfhrentals.sc.egov.usda.gov/RDMFHRentals/projectservlet?cnty=069&amp;st=12; https://affordablehousingonline.com/housing-search/Florida/Leesburg/Pepper-Tree-Apts-II/10104710; https://affordablehousingonline.com/housing-search/Florida/Leesburg</t>
+          <t>https://www.sumtercountyfl.gov/246/Rental-Assistance-Resources; https://www.sumtercountyfl.gov/DocumentCenter/View/29964/Sumter-County-Multifamily-Analysis-Final-Version-06202018; https://sumtercountyfl.gov/246/Rental-Assistance-Resources; https://affordablehousingonline.com/housing-search/Florida/Bushnell/Bushnell-Garden-Apartments/10000207; https://www.lowincomehousing.us/FL/bushnell.html</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -24642,7 +24642,7 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Listed on USDA Rural Development Lake County property list.</t>
+          <t>Outside primary city list but near the target areas and listed by Sumter County as rental assistance provider. | Bushnell Garden Apartments - 352-793-4838</t>
         </is>
       </c>
     </row>

</xml_diff>